<commit_message>
fix: comment garbled + womens monthly target
</commit_message>
<xml_diff>
--- a/2026WB年规进度.xlsx
+++ b/2026WB年规进度.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="13380" activeTab="4"/>
+    <workbookView windowWidth="29868" windowHeight="13380"/>
   </bookViews>
   <sheets>
     <sheet name="毛立新" sheetId="1" r:id="rId1"/>
@@ -22613,7 +22613,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1054e69f-2f7a-4a23-afbd-3884b513e0ca}</x14:id>
+          <x14:id>{a016abcd-22d4-466d-8c95-677345e91d28}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22627,7 +22627,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{981c03dd-b5a3-41cd-91dd-5119ccc55c8b}</x14:id>
+          <x14:id>{6fe96348-2dfb-4928-9319-a7a9eed56793}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22641,7 +22641,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4ce2367b-1d99-4641-9b75-829f18893eaa}</x14:id>
+          <x14:id>{6502992b-89dc-416c-bbb2-ede50ac97beb}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22655,7 +22655,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5d571f6a-7950-4e5b-bed7-2d2a5f756495}</x14:id>
+          <x14:id>{a2fde2db-8a92-4d62-bb49-10c10f0f0caf}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22669,7 +22669,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{243de982-267f-4d7a-b0a3-c95ea3da5294}</x14:id>
+          <x14:id>{e4ccbbdb-773d-4855-b141-d8d5a1317f3f}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22683,7 +22683,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{e00ce940-ae50-4135-9fb3-42bd080a3abd}</x14:id>
+          <x14:id>{626854b4-4e4b-4834-aecb-3af61ce6a0ce}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22697,7 +22697,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{87dbb917-8afa-4cd8-8d01-9e47c90c8995}</x14:id>
+          <x14:id>{7e549c1a-e68b-4869-85ba-3d9890529bd2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22711,7 +22711,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{663f5af0-d7a5-49db-add2-8885af59a442}</x14:id>
+          <x14:id>{2543ade4-5e01-47e9-b848-c030380cb77f}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22725,7 +22725,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d36a9388-56cb-48be-9428-a545eb9849fb}</x14:id>
+          <x14:id>{6b744297-fcbc-4411-b311-b775b9802b5f}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22739,7 +22739,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{50489279-4cd9-4363-ba4e-1d3ad47a71cd}</x14:id>
+          <x14:id>{343d1f63-ed2a-45d7-9051-aa7c1564c26f}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22753,7 +22753,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4b9ea658-3e4f-4d39-818e-5e76a3d2d72e}</x14:id>
+          <x14:id>{af2f9fdf-7b5a-4972-a9ab-5b7d2d56451c}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22767,7 +22767,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9b3600b1-889a-4d63-af5d-12086c640a8f}</x14:id>
+          <x14:id>{517fc391-1d6b-4c01-aa2e-4b74e8504069}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22781,7 +22781,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{34b913d2-4d09-44ef-9ac4-f54fcafdecb7}</x14:id>
+          <x14:id>{c18c4523-ca3b-4339-942b-e3ba14fc0e3a}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22803,7 +22803,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{a3b1401f-9a89-4373-a055-936d0a224c9d}</x14:id>
+          <x14:id>{b13cc5a6-c7ed-4955-a6e0-a3b6be7982d0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22833,7 +22833,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{da948d02-b053-41a1-b468-7dbd2645871a}</x14:id>
+          <x14:id>{654b787c-0f28-45d1-906b-1bd22693177d}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22863,7 +22863,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3fe7fed2-b1cf-4012-8c20-ba6118ea55ba}</x14:id>
+          <x14:id>{1701f32b-2a7a-4684-ad8a-c0ead8e16efc}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22893,7 +22893,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{a498e1ff-c4ab-4f5c-b462-1b1258df0b2b}</x14:id>
+          <x14:id>{a4bbfc25-3dee-4fad-a621-0194c12ce8b1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22923,7 +22923,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{fb436dce-c161-4296-83ce-2fb88b8b944b}</x14:id>
+          <x14:id>{a694973c-93d5-41d0-bb80-55cbcca12318}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22953,7 +22953,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{29e276b4-e426-4cb1-b741-f5ad16f817f1}</x14:id>
+          <x14:id>{18dd4a86-b6d1-40c9-b28b-4cd3723f1739}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22983,7 +22983,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7483cd84-eb09-458c-b80b-4bf502db0fe9}</x14:id>
+          <x14:id>{909b4df7-a3a6-4d7b-945a-95fd9d5ad9c0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23013,7 +23013,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{acfdff71-e3ad-48c5-b6da-dc28d4114659}</x14:id>
+          <x14:id>{0dc4fcbc-84b9-44ec-93d6-76ca51215997}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23035,7 +23035,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{647570c6-44b4-4f68-a894-4d52241e04dc}</x14:id>
+          <x14:id>{55bbc241-df66-4a25-852e-1ee954dcea21}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23057,7 +23057,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{137ec496-f13c-46ee-8243-33d7cc20497b}</x14:id>
+          <x14:id>{b83ec02a-a3b2-4ff3-9717-9cf1c077da9a}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23079,7 +23079,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{477bbc9b-60f1-49c6-add4-eb44ecde81f6}</x14:id>
+          <x14:id>{c79266ae-d78e-4e8a-b5a4-2f3cd6648cc9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23101,7 +23101,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{a3c5cca8-c0a9-4c7d-b729-ad3ed0105303}</x14:id>
+          <x14:id>{ebaa7727-d357-4647-815c-b32c7cbd3ff3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23123,7 +23123,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{c4db7b94-317d-4d27-b7f7-27d224e8099f}</x14:id>
+          <x14:id>{767194b9-c723-4ee1-a7c2-65e1c3befab8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23145,7 +23145,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4a0a589f-5e6b-438d-9c25-a69a16353ad0}</x14:id>
+          <x14:id>{8b73abb9-83fd-4667-9cbb-e4a293f10223}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23167,7 +23167,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{733aae13-c8a1-41be-baee-0e45846e41fb}</x14:id>
+          <x14:id>{8a1c5415-fdae-40e2-865c-d97e7fed5b15}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23189,7 +23189,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0f084c0c-61b1-412a-97ad-5b3eee9c37aa}</x14:id>
+          <x14:id>{19a10da5-7bf5-42f8-967e-69d37686fb4e}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23211,7 +23211,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5c0d6a4d-a67c-474e-84aa-c20c51621ac9}</x14:id>
+          <x14:id>{dd6d3ddd-be5a-4043-ae26-46f0740f9223}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23233,7 +23233,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{78fd8f19-b9e0-4f84-85f8-136e50cfb38b}</x14:id>
+          <x14:id>{7fa22bd8-893d-4b87-9450-94715ccc637c}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23255,7 +23255,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{bd90acee-1578-41bc-ac97-5a562ba27e69}</x14:id>
+          <x14:id>{f798e696-c6ee-4f39-b2b3-fbe48e047023}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23277,7 +23277,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{90ee968d-a976-45ba-b327-e67fdbb27f5c}</x14:id>
+          <x14:id>{81ce6cfa-5cc6-475a-b050-4850cb980e67}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23296,7 +23296,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1054e69f-2f7a-4a23-afbd-3884b513e0ca}">
+          <x14:cfRule type="dataBar" id="{a016abcd-22d4-466d-8c95-677345e91d28}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23309,7 +23309,7 @@
           <xm:sqref>C8:O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{981c03dd-b5a3-41cd-91dd-5119ccc55c8b}">
+          <x14:cfRule type="dataBar" id="{6fe96348-2dfb-4928-9319-a7a9eed56793}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23322,7 +23322,7 @@
           <xm:sqref>C12:O12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4ce2367b-1d99-4641-9b75-829f18893eaa}">
+          <x14:cfRule type="dataBar" id="{6502992b-89dc-416c-bbb2-ede50ac97beb}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23335,7 +23335,7 @@
           <xm:sqref>C16:O16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5d571f6a-7950-4e5b-bed7-2d2a5f756495}">
+          <x14:cfRule type="dataBar" id="{a2fde2db-8a92-4d62-bb49-10c10f0f0caf}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23348,7 +23348,7 @@
           <xm:sqref>C20:O20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{243de982-267f-4d7a-b0a3-c95ea3da5294}">
+          <x14:cfRule type="dataBar" id="{e4ccbbdb-773d-4855-b141-d8d5a1317f3f}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23361,7 +23361,7 @@
           <xm:sqref>C24:O24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{e00ce940-ae50-4135-9fb3-42bd080a3abd}">
+          <x14:cfRule type="dataBar" id="{626854b4-4e4b-4834-aecb-3af61ce6a0ce}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23374,7 +23374,7 @@
           <xm:sqref>C27:O27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{87dbb917-8afa-4cd8-8d01-9e47c90c8995}">
+          <x14:cfRule type="dataBar" id="{7e549c1a-e68b-4869-85ba-3d9890529bd2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23387,7 +23387,7 @@
           <xm:sqref>C36:O36</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{663f5af0-d7a5-49db-add2-8885af59a442}">
+          <x14:cfRule type="dataBar" id="{2543ade4-5e01-47e9-b848-c030380cb77f}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23400,7 +23400,7 @@
           <xm:sqref>C44:O44</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d36a9388-56cb-48be-9428-a545eb9849fb}">
+          <x14:cfRule type="dataBar" id="{6b744297-fcbc-4411-b311-b775b9802b5f}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23413,7 +23413,7 @@
           <xm:sqref>C52:O52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{50489279-4cd9-4363-ba4e-1d3ad47a71cd}">
+          <x14:cfRule type="dataBar" id="{343d1f63-ed2a-45d7-9051-aa7c1564c26f}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23426,7 +23426,7 @@
           <xm:sqref>C60:O60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4b9ea658-3e4f-4d39-818e-5e76a3d2d72e}">
+          <x14:cfRule type="dataBar" id="{af2f9fdf-7b5a-4972-a9ab-5b7d2d56451c}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23439,7 +23439,7 @@
           <xm:sqref>C68:O68</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9b3600b1-889a-4d63-af5d-12086c640a8f}">
+          <x14:cfRule type="dataBar" id="{517fc391-1d6b-4c01-aa2e-4b74e8504069}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23452,7 +23452,7 @@
           <xm:sqref>C76:O76</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{34b913d2-4d09-44ef-9ac4-f54fcafdecb7}">
+          <x14:cfRule type="dataBar" id="{c18c4523-ca3b-4339-942b-e3ba14fc0e3a}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23465,7 +23465,7 @@
           <xm:sqref>C132:O132</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{a3b1401f-9a89-4373-a055-936d0a224c9d}">
+          <x14:cfRule type="dataBar" id="{b13cc5a6-c7ed-4955-a6e0-a3b6be7982d0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23478,7 +23478,7 @@
           <xm:sqref>C26:O26 D27:N27 C28:O28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{da948d02-b053-41a1-b468-7dbd2645871a}">
+          <x14:cfRule type="dataBar" id="{654b787c-0f28-45d1-906b-1bd22693177d}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23491,7 +23491,7 @@
           <xm:sqref>C35:O35 D36:N36 C37:O37</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3fe7fed2-b1cf-4012-8c20-ba6118ea55ba}">
+          <x14:cfRule type="dataBar" id="{1701f32b-2a7a-4684-ad8a-c0ead8e16efc}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23504,7 +23504,7 @@
           <xm:sqref>C43:O43 D44:N44 C45:O45</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{a498e1ff-c4ab-4f5c-b462-1b1258df0b2b}">
+          <x14:cfRule type="dataBar" id="{a4bbfc25-3dee-4fad-a621-0194c12ce8b1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23517,7 +23517,7 @@
           <xm:sqref>C51:O51 D52:N52 C53:O53</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{fb436dce-c161-4296-83ce-2fb88b8b944b}">
+          <x14:cfRule type="dataBar" id="{a694973c-93d5-41d0-bb80-55cbcca12318}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23530,7 +23530,7 @@
           <xm:sqref>C59:O59 D60:N60 C61:O61</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{29e276b4-e426-4cb1-b741-f5ad16f817f1}">
+          <x14:cfRule type="dataBar" id="{18dd4a86-b6d1-40c9-b28b-4cd3723f1739}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23543,7 +23543,7 @@
           <xm:sqref>C67:O67 D68:N68 C69:O69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7483cd84-eb09-458c-b80b-4bf502db0fe9}">
+          <x14:cfRule type="dataBar" id="{909b4df7-a3a6-4d7b-945a-95fd9d5ad9c0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23556,7 +23556,7 @@
           <xm:sqref>C75:O75 D76:N76 C77:O77</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{acfdff71-e3ad-48c5-b6da-dc28d4114659}">
+          <x14:cfRule type="dataBar" id="{0dc4fcbc-84b9-44ec-93d6-76ca51215997}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23569,7 +23569,7 @@
           <xm:sqref>C83:N83 D84:N84 C85:O85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{647570c6-44b4-4f68-a894-4d52241e04dc}">
+          <x14:cfRule type="dataBar" id="{55bbc241-df66-4a25-852e-1ee954dcea21}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23582,7 +23582,7 @@
           <xm:sqref>C84:O84 D85:N85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{137ec496-f13c-46ee-8243-33d7cc20497b}">
+          <x14:cfRule type="dataBar" id="{b83ec02a-a3b2-4ff3-9717-9cf1c077da9a}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23595,7 +23595,7 @@
           <xm:sqref>C91:N91 D92:N92 C93:O93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{477bbc9b-60f1-49c6-add4-eb44ecde81f6}">
+          <x14:cfRule type="dataBar" id="{c79266ae-d78e-4e8a-b5a4-2f3cd6648cc9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23608,7 +23608,7 @@
           <xm:sqref>C92:O92 D93:N93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{a3c5cca8-c0a9-4c7d-b729-ad3ed0105303}">
+          <x14:cfRule type="dataBar" id="{ebaa7727-d357-4647-815c-b32c7cbd3ff3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23621,7 +23621,7 @@
           <xm:sqref>C99:N99 D100:N100 C101:O101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{c4db7b94-317d-4d27-b7f7-27d224e8099f}">
+          <x14:cfRule type="dataBar" id="{767194b9-c723-4ee1-a7c2-65e1c3befab8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23634,7 +23634,7 @@
           <xm:sqref>C100:O100 D101:N101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4a0a589f-5e6b-438d-9c25-a69a16353ad0}">
+          <x14:cfRule type="dataBar" id="{8b73abb9-83fd-4667-9cbb-e4a293f10223}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23647,7 +23647,7 @@
           <xm:sqref>C107:N107 D108:N108 C109:O109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{733aae13-c8a1-41be-baee-0e45846e41fb}">
+          <x14:cfRule type="dataBar" id="{8a1c5415-fdae-40e2-865c-d97e7fed5b15}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23660,7 +23660,7 @@
           <xm:sqref>C108:O108 D109:N109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0f084c0c-61b1-412a-97ad-5b3eee9c37aa}">
+          <x14:cfRule type="dataBar" id="{19a10da5-7bf5-42f8-967e-69d37686fb4e}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23673,7 +23673,7 @@
           <xm:sqref>C115:N115 D116:N116 C117:O117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5c0d6a4d-a67c-474e-84aa-c20c51621ac9}">
+          <x14:cfRule type="dataBar" id="{dd6d3ddd-be5a-4043-ae26-46f0740f9223}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23686,7 +23686,7 @@
           <xm:sqref>C116:O116 D117:N117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{78fd8f19-b9e0-4f84-85f8-136e50cfb38b}">
+          <x14:cfRule type="dataBar" id="{7fa22bd8-893d-4b87-9450-94715ccc637c}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23699,7 +23699,7 @@
           <xm:sqref>C123:N123 D124:N124 C125:O125</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{bd90acee-1578-41bc-ac97-5a562ba27e69}">
+          <x14:cfRule type="dataBar" id="{f798e696-c6ee-4f39-b2b3-fbe48e047023}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -23712,7 +23712,7 @@
           <xm:sqref>C124:O124 D125:N125</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{90ee968d-a976-45ba-b327-e67fdbb27f5c}">
+          <x14:cfRule type="dataBar" id="{81ce6cfa-5cc6-475a-b050-4850cb980e67}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -34276,7 +34276,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{37b4cf6a-1808-4072-a0a7-ecbff381979c}</x14:id>
+          <x14:id>{65462c0c-7b84-4fbe-b98e-ff79d2c637fe}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34290,7 +34290,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{be9fe18a-c2d8-488a-b536-b1c77c15f7d5}</x14:id>
+          <x14:id>{36bc6679-be8c-4692-be64-b765b9623819}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34304,7 +34304,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{e71aabf7-ef0c-4b6e-961c-40d63fbe8141}</x14:id>
+          <x14:id>{c2ba36c0-8c43-4dd3-a86d-af3a09842750}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34318,7 +34318,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{b39c01d6-657b-4257-9405-33eb62f32816}</x14:id>
+          <x14:id>{7cff423f-95a6-4dda-8da4-62f83672ddc4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34332,7 +34332,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{610462a8-73a7-479f-9ee1-7d28bc2071fc}</x14:id>
+          <x14:id>{191764a0-8d30-41ec-8b5d-2acbcb8a79bb}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34346,7 +34346,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{add3203e-8fdc-4a24-9a4b-a2a87c69e149}</x14:id>
+          <x14:id>{4251c6c6-7098-4a1d-90b2-35b1dc5e887b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34366,7 +34366,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{028261ba-7800-477d-99d4-efc900c4723b}</x14:id>
+          <x14:id>{a680dfff-54fe-4eda-8423-940449a60f07}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34380,7 +34380,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{37397be4-311b-469d-80cc-a5357eac4c7a}</x14:id>
+          <x14:id>{cd793ddd-1034-4dba-a943-39fa46bacb6a}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34394,7 +34394,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1ae182f9-8190-4f87-a4ed-041ec8f81f7d}</x14:id>
+          <x14:id>{b1e3eaeb-8c2f-4a8b-bbd1-d83cc56074c0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34408,7 +34408,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2ba0824c-f52b-4dcc-8347-ae440ee6da19}</x14:id>
+          <x14:id>{eab9e69c-2be1-44cb-9d34-1dc9dc7c7359}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34422,7 +34422,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{13b6d504-c4ce-49a5-a654-7abb013a5d8c}</x14:id>
+          <x14:id>{66a37adb-046b-4a13-b51a-e67b1c2d3784}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34436,7 +34436,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{f98fea20-7d7a-465e-b4ac-dfe08f5af8be}</x14:id>
+          <x14:id>{98de2829-249e-4add-ad49-1c6dbca1b224}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34458,7 +34458,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{794d11de-a650-4e12-b0eb-bb54e416e9df}</x14:id>
+          <x14:id>{a33eca60-86f4-4f42-80ae-858301d34a96}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34488,7 +34488,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{58910e22-0afa-4cb6-ba8a-4a132830ce08}</x14:id>
+          <x14:id>{24e2c323-81e6-4931-91b2-277e1620a31c}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34518,7 +34518,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{85f59fcc-63be-4732-a6a8-8a9c797f6151}</x14:id>
+          <x14:id>{fb85fc6e-9983-481c-81d3-283503624b44}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34548,7 +34548,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7eb57a5c-7124-43a8-bddd-37f7a11e15c2}</x14:id>
+          <x14:id>{8880b95d-ba92-4496-b81e-ac2e9eb0cbc7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34578,7 +34578,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{09507472-92d1-48ec-a69b-7f7d44c53a6e}</x14:id>
+          <x14:id>{fc7c09cf-5626-491d-bc29-11310e59de92}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34608,7 +34608,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3c3ea18b-549f-4967-a25c-af7b142030e6}</x14:id>
+          <x14:id>{de349661-009a-4421-9e42-0f0908b06e01}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34630,7 +34630,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{b36236e6-81ac-4613-a6b0-449683f70c79}</x14:id>
+          <x14:id>{0e9a0a42-1380-431c-842b-02bf42abf4cd}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34652,7 +34652,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8170bdcc-317b-4bb7-b230-83e6f842a24c}</x14:id>
+          <x14:id>{57b2f5c6-fe24-4f90-ad16-15bca24eb9c5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34674,7 +34674,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{a14663ef-6ca3-489a-8764-dd64bea45c40}</x14:id>
+          <x14:id>{81341fb8-65d3-440d-853d-829e2890b637}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34696,7 +34696,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d52088cc-74b1-417b-b96a-e1482f5bf465}</x14:id>
+          <x14:id>{edad3efa-394b-4cc7-b5ae-2b2d102fb2cb}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34718,7 +34718,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{c0faf253-cc75-4a5c-a754-7281e807c8e4}</x14:id>
+          <x14:id>{0dfc7044-a09e-4b91-a2e5-cb5a50bd90f5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34740,7 +34740,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d65e3b33-aeae-4ee7-91bb-f78580f39f29}</x14:id>
+          <x14:id>{88b5b45f-8848-4e70-a0fb-8ed67ef4fbc2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34762,7 +34762,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{52c066db-a5d6-4898-a5c6-ede2ea23211d}</x14:id>
+          <x14:id>{e9b3a736-511d-4960-bba5-b5d3328736b2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34784,7 +34784,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{241d21de-c337-4d06-83ee-516268cb0f21}</x14:id>
+          <x14:id>{1711f887-3478-46db-a648-3a1c216995e0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34806,7 +34806,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{806fdb81-a199-4bc1-93c3-403474048fa2}</x14:id>
+          <x14:id>{8d85ff60-e1c9-4c5a-af4d-946707eafb02}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34828,7 +34828,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{dccdf48c-f693-46a3-a165-831c4a31e083}</x14:id>
+          <x14:id>{04058a32-8600-4a9c-88f6-a92c2f236ae6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34850,7 +34850,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{88a7a9a8-b902-4f12-b27d-7b37b02b2ee6}</x14:id>
+          <x14:id>{bf27e5bb-8461-4e74-8b0e-52cc4e86506c}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34872,7 +34872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{c2691c27-f02d-49f7-8b65-0f2921a68e4c}</x14:id>
+          <x14:id>{d86bb071-e9e1-4ff2-aaf4-fba822caca0b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34894,7 +34894,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{fcd04a44-8c24-47b7-ab63-6980a58ca34d}</x14:id>
+          <x14:id>{9e8fb8b3-e4fc-4838-9443-95a680cca7ad}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34916,7 +34916,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{cebd219a-8fcc-488c-9747-329f36f12195}</x14:id>
+          <x14:id>{65a22b99-8280-47cc-a2ca-1bb6aaef71d3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -34935,7 +34935,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{37b4cf6a-1808-4072-a0a7-ecbff381979c}">
+          <x14:cfRule type="dataBar" id="{65462c0c-7b84-4fbe-b98e-ff79d2c637fe}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -34948,7 +34948,7 @@
           <xm:sqref>C8:O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{be9fe18a-c2d8-488a-b536-b1c77c15f7d5}">
+          <x14:cfRule type="dataBar" id="{36bc6679-be8c-4692-be64-b765b9623819}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -34961,7 +34961,7 @@
           <xm:sqref>C12:O12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{e71aabf7-ef0c-4b6e-961c-40d63fbe8141}">
+          <x14:cfRule type="dataBar" id="{c2ba36c0-8c43-4dd3-a86d-af3a09842750}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -34974,7 +34974,7 @@
           <xm:sqref>C16:O16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{b39c01d6-657b-4257-9405-33eb62f32816}">
+          <x14:cfRule type="dataBar" id="{7cff423f-95a6-4dda-8da4-62f83672ddc4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -34987,7 +34987,7 @@
           <xm:sqref>C20:O20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{610462a8-73a7-479f-9ee1-7d28bc2071fc}">
+          <x14:cfRule type="dataBar" id="{191764a0-8d30-41ec-8b5d-2acbcb8a79bb}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35000,7 +35000,7 @@
           <xm:sqref>C24:O24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{add3203e-8fdc-4a24-9a4b-a2a87c69e149}">
+          <x14:cfRule type="dataBar" id="{4251c6c6-7098-4a1d-90b2-35b1dc5e887b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35013,7 +35013,7 @@
           <xm:sqref>O26</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{028261ba-7800-477d-99d4-efc900c4723b}">
+          <x14:cfRule type="dataBar" id="{a680dfff-54fe-4eda-8423-940449a60f07}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35026,7 +35026,7 @@
           <xm:sqref>C27:O27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{37397be4-311b-469d-80cc-a5357eac4c7a}">
+          <x14:cfRule type="dataBar" id="{cd793ddd-1034-4dba-a943-39fa46bacb6a}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35039,7 +35039,7 @@
           <xm:sqref>C36:O36</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1ae182f9-8190-4f87-a4ed-041ec8f81f7d}">
+          <x14:cfRule type="dataBar" id="{b1e3eaeb-8c2f-4a8b-bbd1-d83cc56074c0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35052,7 +35052,7 @@
           <xm:sqref>C44:O44</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2ba0824c-f52b-4dcc-8347-ae440ee6da19}">
+          <x14:cfRule type="dataBar" id="{eab9e69c-2be1-44cb-9d34-1dc9dc7c7359}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35065,7 +35065,7 @@
           <xm:sqref>C52:O52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{13b6d504-c4ce-49a5-a654-7abb013a5d8c}">
+          <x14:cfRule type="dataBar" id="{66a37adb-046b-4a13-b51a-e67b1c2d3784}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35078,7 +35078,7 @@
           <xm:sqref>C60:O60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{f98fea20-7d7a-465e-b4ac-dfe08f5af8be}">
+          <x14:cfRule type="dataBar" id="{98de2829-249e-4add-ad49-1c6dbca1b224}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35091,7 +35091,7 @@
           <xm:sqref>C124:O124</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{794d11de-a650-4e12-b0eb-bb54e416e9df}">
+          <x14:cfRule type="dataBar" id="{a33eca60-86f4-4f42-80ae-858301d34a96}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35104,7 +35104,7 @@
           <xm:sqref>C26:N26 D27:N27 C28:O28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{58910e22-0afa-4cb6-ba8a-4a132830ce08}">
+          <x14:cfRule type="dataBar" id="{24e2c323-81e6-4931-91b2-277e1620a31c}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35117,7 +35117,7 @@
           <xm:sqref>C35:N35 D36:N36 C37:O37</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{85f59fcc-63be-4732-a6a8-8a9c797f6151}">
+          <x14:cfRule type="dataBar" id="{fb85fc6e-9983-481c-81d3-283503624b44}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35130,7 +35130,7 @@
           <xm:sqref>C43:N43 D44:N44 C45:O45</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7eb57a5c-7124-43a8-bddd-37f7a11e15c2}">
+          <x14:cfRule type="dataBar" id="{8880b95d-ba92-4496-b81e-ac2e9eb0cbc7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35143,7 +35143,7 @@
           <xm:sqref>C51:N51 D52:N52 C53:O53</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{09507472-92d1-48ec-a69b-7f7d44c53a6e}">
+          <x14:cfRule type="dataBar" id="{fc7c09cf-5626-491d-bc29-11310e59de92}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35156,7 +35156,7 @@
           <xm:sqref>C59:N59 D60:N60 C61:O61</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3c3ea18b-549f-4967-a25c-af7b142030e6}">
+          <x14:cfRule type="dataBar" id="{de349661-009a-4421-9e42-0f0908b06e01}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35169,7 +35169,7 @@
           <xm:sqref>C67:N67 D68:N68 C69:O69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{b36236e6-81ac-4613-a6b0-449683f70c79}">
+          <x14:cfRule type="dataBar" id="{0e9a0a42-1380-431c-842b-02bf42abf4cd}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35182,7 +35182,7 @@
           <xm:sqref>C68:O68 D69:N69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8170bdcc-317b-4bb7-b230-83e6f842a24c}">
+          <x14:cfRule type="dataBar" id="{57b2f5c6-fe24-4f90-ad16-15bca24eb9c5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35195,7 +35195,7 @@
           <xm:sqref>C75:N75 D76:N76 C77:O77</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{a14663ef-6ca3-489a-8764-dd64bea45c40}">
+          <x14:cfRule type="dataBar" id="{81341fb8-65d3-440d-853d-829e2890b637}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35208,7 +35208,7 @@
           <xm:sqref>C76:O76 D77:N77</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d52088cc-74b1-417b-b96a-e1482f5bf465}">
+          <x14:cfRule type="dataBar" id="{edad3efa-394b-4cc7-b5ae-2b2d102fb2cb}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35221,7 +35221,7 @@
           <xm:sqref>C83:N83 D84:N84 C85:O85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{c0faf253-cc75-4a5c-a754-7281e807c8e4}">
+          <x14:cfRule type="dataBar" id="{0dfc7044-a09e-4b91-a2e5-cb5a50bd90f5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35234,7 +35234,7 @@
           <xm:sqref>C84:O84 D85:N85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d65e3b33-aeae-4ee7-91bb-f78580f39f29}">
+          <x14:cfRule type="dataBar" id="{88b5b45f-8848-4e70-a0fb-8ed67ef4fbc2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35247,7 +35247,7 @@
           <xm:sqref>C91:N91 D92:N92 C93:O93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{52c066db-a5d6-4898-a5c6-ede2ea23211d}">
+          <x14:cfRule type="dataBar" id="{e9b3a736-511d-4960-bba5-b5d3328736b2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35260,7 +35260,7 @@
           <xm:sqref>C92:O92 D93:N93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{241d21de-c337-4d06-83ee-516268cb0f21}">
+          <x14:cfRule type="dataBar" id="{1711f887-3478-46db-a648-3a1c216995e0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35273,7 +35273,7 @@
           <xm:sqref>C99:N99 D100:N100 C101:O101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{806fdb81-a199-4bc1-93c3-403474048fa2}">
+          <x14:cfRule type="dataBar" id="{8d85ff60-e1c9-4c5a-af4d-946707eafb02}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35286,7 +35286,7 @@
           <xm:sqref>C100:O100 D101:N101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{dccdf48c-f693-46a3-a165-831c4a31e083}">
+          <x14:cfRule type="dataBar" id="{04058a32-8600-4a9c-88f6-a92c2f236ae6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35299,7 +35299,7 @@
           <xm:sqref>C107:N107 D108:N108 C109:O109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{88a7a9a8-b902-4f12-b27d-7b37b02b2ee6}">
+          <x14:cfRule type="dataBar" id="{bf27e5bb-8461-4e74-8b0e-52cc4e86506c}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35312,7 +35312,7 @@
           <xm:sqref>C108:O108 D109:N109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{c2691c27-f02d-49f7-8b65-0f2921a68e4c}">
+          <x14:cfRule type="dataBar" id="{d86bb071-e9e1-4ff2-aaf4-fba822caca0b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35325,7 +35325,7 @@
           <xm:sqref>C115:N115 D116:N116 C117:O117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{fcd04a44-8c24-47b7-ab63-6980a58ca34d}">
+          <x14:cfRule type="dataBar" id="{9e8fb8b3-e4fc-4838-9443-95a680cca7ad}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -35338,7 +35338,7 @@
           <xm:sqref>C116:O116 D117:N117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{cebd219a-8fcc-488c-9747-329f36f12195}">
+          <x14:cfRule type="dataBar" id="{65a22b99-8280-47cc-a2ca-1bb6aaef71d3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -40483,7 +40483,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ca5a9f72-d66d-49c0-a23e-6ca9f49a3bf9}</x14:id>
+          <x14:id>{99f1a2b3-c306-4cb7-8d49-ccf10fc43518}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -40494,7 +40494,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ca5a9f72-d66d-49c0-a23e-6ca9f49a3bf9}">
+          <x14:cfRule type="dataBar" id="{99f1a2b3-c306-4cb7-8d49-ccf10fc43518}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
fix: build_data_women.py 同步生成 data-detail-women.js，修复女装数据不刷新
</commit_message>
<xml_diff>
--- a/2026WB年规进度.xlsx
+++ b/2026WB年规进度.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="13380" activeTab="4"/>
+    <workbookView windowWidth="29868" windowHeight="13380" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="毛立新" sheetId="1" r:id="rId1"/>
@@ -23231,7 +23231,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{12705517-a1ac-4af3-9c47-dffcbd884c69}</x14:id>
+          <x14:id>{a0bf4642-49d5-4902-863b-b161d3ac2e43}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23245,7 +23245,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0e1a063c-cfc4-4370-b5f5-e3d78bae61f4}</x14:id>
+          <x14:id>{c73feab8-9790-423c-815a-8d6d80400539}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23259,7 +23259,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6d90900b-c779-4f2d-8b04-1d186ac211c5}</x14:id>
+          <x14:id>{a22acc92-8d40-489f-905e-7dc2e21ad47a}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23273,7 +23273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{538c34ba-3fe1-4246-a987-1e6331b69a84}</x14:id>
+          <x14:id>{bb2ba546-383a-408d-9258-176c2a4c9cc5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23287,7 +23287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4d191783-513b-4681-a0e0-1da47cce2353}</x14:id>
+          <x14:id>{1911f09d-a918-424f-8b83-38061cd6a8c8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23301,7 +23301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{a6de7bd0-e68f-4f22-9a4b-52508451c1bf}</x14:id>
+          <x14:id>{64fa7fee-d917-4de0-9f2c-445b0d3c0cea}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23315,7 +23315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2f855105-ca70-48e9-bb22-0a86855ee54f}</x14:id>
+          <x14:id>{599f4c3d-84b4-43cf-9e7e-b4e2885abd59}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23329,7 +23329,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{bbf82617-38a1-4e97-9e72-eb5a0c3bdb92}</x14:id>
+          <x14:id>{c327917d-ddae-4604-a315-4ee53f7f857f}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23349,7 +23349,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{60698893-4c65-4d50-af79-65729be2c6b5}</x14:id>
+          <x14:id>{278383ae-5d9e-4ba1-9eab-ce54cad1a3e3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23377,7 +23377,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0d3ac796-bdc0-45d4-8882-852723bc1c17}</x14:id>
+          <x14:id>{d40bccc4-781f-478a-91c5-afe98f15aeaf}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23397,7 +23397,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{261db87c-1e88-4ec8-bfd4-f9ff58e6ab69}</x14:id>
+          <x14:id>{e0e54f1a-610f-44d6-9a42-75de4393b59c}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23425,7 +23425,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{c7327550-3ab0-47f9-87ae-ebc7daa8c728}</x14:id>
+          <x14:id>{55f821aa-6302-4bc2-9058-472ebe7b94cd}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23445,7 +23445,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{cd911691-1116-42fe-bc53-67b1c0267f3b}</x14:id>
+          <x14:id>{d3866566-82c4-41d8-a6c1-357419a7e181}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23473,7 +23473,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{488d3490-7eae-4875-a20c-b6e313a891f8}</x14:id>
+          <x14:id>{041a0567-316c-4c6c-b59c-04cc0a128409}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23493,7 +23493,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d32d3730-c799-495f-ab3f-368a55c0587b}</x14:id>
+          <x14:id>{13edfe20-6c42-4c8d-af9d-9e2ec69aeaae}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23521,7 +23521,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{917a537d-9e87-4c62-970e-2a3208257cff}</x14:id>
+          <x14:id>{3145c08a-d8f1-4263-b847-f6ca27453b95}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23541,7 +23541,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{a0816f8a-cf6d-4ed6-be91-32fb8a7baa2b}</x14:id>
+          <x14:id>{cf2b4519-b2fb-4cc8-a377-bc0c000da78d}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23569,7 +23569,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{46e4e21c-a7ec-4379-8b05-59f6f8733a0d}</x14:id>
+          <x14:id>{d54ffcba-f4e0-4a29-a988-b266d9749fea}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23631,7 +23631,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{62b58732-fa75-415f-ae8c-e06cbb39486c}</x14:id>
+          <x14:id>{135f8d21-d3d4-4de5-ae41-c1e1d6d183bb}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23661,7 +23661,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{71e9fd37-0a20-44b6-bc97-8c3bc7b56d3c}</x14:id>
+          <x14:id>{7f5dccef-1bfb-492c-810e-be66cdfe0aaf}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23683,7 +23683,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1f554681-6d53-4dfd-9c51-909b0684a3a5}</x14:id>
+          <x14:id>{c23207e8-182b-40b1-9bcb-03876318e320}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23703,7 +23703,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{53a4cf40-caa0-4fba-a9ce-286287c1ff0d}</x14:id>
+          <x14:id>{aaac129a-cbca-490b-b1be-888331b9f70a}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23725,7 +23725,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7257bc84-0606-4596-9096-c367964143e1}</x14:id>
+          <x14:id>{c8cba163-b45a-4e26-a0ba-9a227b6f777a}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23745,7 +23745,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{b53cb82c-b426-442c-9227-d43032399732}</x14:id>
+          <x14:id>{d7451388-b77c-4e86-8099-85feb02bc130}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23767,7 +23767,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{b670fcd2-c030-4af4-a7c8-fa413a7d467a}</x14:id>
+          <x14:id>{f46ba46a-a72d-4c82-bc6b-466cc725a101}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23787,7 +23787,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3b8e60aa-309d-4e94-9e38-064c7c48539b}</x14:id>
+          <x14:id>{596bc0b3-802d-4592-94cc-81c20fd68aa5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23809,7 +23809,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8004c6e5-6aef-472d-9deb-d7bb3eb0a282}</x14:id>
+          <x14:id>{62f6e842-9461-4335-ab10-020b94a0c86c}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23829,7 +23829,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8514cc6f-c463-4734-8c35-aebf1ed97435}</x14:id>
+          <x14:id>{333ac094-d46f-4ba5-aa34-e2c597442e72}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23857,7 +23857,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{a79d2cca-63f7-4381-b276-ddc721ebedda}</x14:id>
+          <x14:id>{e00d3cdb-d6b7-493d-a01d-92157d3877d2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23871,7 +23871,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{830a7799-181e-4617-84cd-a83d5c0c5070}</x14:id>
+          <x14:id>{1efa4371-2280-4078-b7a9-4bed4b5c3ad8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23901,7 +23901,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d533caa9-ee38-4a38-89c9-b295f24de74e}</x14:id>
+          <x14:id>{afa2d65e-8b95-482b-9232-62e59aa41830}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23923,7 +23923,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{af742c9d-636f-4fff-ac6a-7f9c7f3c7037}</x14:id>
+          <x14:id>{26e8731e-9f2a-41b7-b680-0ccbeee0b679}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23945,7 +23945,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{81f1277b-500d-4e6c-aadd-268bf1ea342a}</x14:id>
+          <x14:id>{3cdc7788-f761-42e3-be98-2218d145b981}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23967,7 +23967,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{e850438a-52e9-4882-a1ef-da02391dd87e}</x14:id>
+          <x14:id>{33a32dd6-7c3d-4131-bff3-5d7a133657f6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23989,7 +23989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3ac28c79-7159-43ed-93c3-5211aa02ceeb}</x14:id>
+          <x14:id>{57339abf-3c6b-4c81-a843-3b96853dd772}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24011,7 +24011,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2e892bd2-e689-47f3-a102-223c279a2883}</x14:id>
+          <x14:id>{c5cc5271-65d0-4a0f-8cee-d2a5303bff74}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24033,7 +24033,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{a7bf0662-6c40-4e21-832f-22511f489591}</x14:id>
+          <x14:id>{26477af8-b059-4a6c-965b-a6f139d7679b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24055,7 +24055,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3baefdbb-4bb1-49bd-a3d7-cd63bcb4e76f}</x14:id>
+          <x14:id>{38415ac6-3eea-4117-b45e-fee9baecd296}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24077,7 +24077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{b197a809-348b-44d9-a999-27a78e001bfc}</x14:id>
+          <x14:id>{160e3e68-d9eb-41ff-a4b9-cf41893e7cd5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24099,7 +24099,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{f4d769d6-5e2c-4223-8934-90e7dffbf419}</x14:id>
+          <x14:id>{cb18ce02-89e7-4e45-b6bf-6c71c8b5ffe8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24121,7 +24121,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8c1fd285-8e9d-444b-a958-7c4598e8275c}</x14:id>
+          <x14:id>{904cf8e6-f644-4be8-b62c-6bc421b3bf03}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24143,7 +24143,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{622dc457-61a6-47ea-9505-488aaa864ee4}</x14:id>
+          <x14:id>{ec21f11a-afe1-4d6c-aac2-cdcf67fc6d02}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24165,7 +24165,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8e4e4590-eeec-47e3-a926-0c76b04861bd}</x14:id>
+          <x14:id>{2dae02d0-c2f2-4046-a497-b9cb14f37060}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24184,7 +24184,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{12705517-a1ac-4af3-9c47-dffcbd884c69}">
+          <x14:cfRule type="dataBar" id="{a0bf4642-49d5-4902-863b-b161d3ac2e43}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24197,7 +24197,7 @@
           <xm:sqref>C8:O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0e1a063c-cfc4-4370-b5f5-e3d78bae61f4}">
+          <x14:cfRule type="dataBar" id="{c73feab8-9790-423c-815a-8d6d80400539}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24210,7 +24210,7 @@
           <xm:sqref>C12:O12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6d90900b-c779-4f2d-8b04-1d186ac211c5}">
+          <x14:cfRule type="dataBar" id="{a22acc92-8d40-489f-905e-7dc2e21ad47a}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24223,7 +24223,7 @@
           <xm:sqref>C16:O16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{538c34ba-3fe1-4246-a987-1e6331b69a84}">
+          <x14:cfRule type="dataBar" id="{bb2ba546-383a-408d-9258-176c2a4c9cc5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24236,7 +24236,7 @@
           <xm:sqref>C20:O20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4d191783-513b-4681-a0e0-1da47cce2353}">
+          <x14:cfRule type="dataBar" id="{1911f09d-a918-424f-8b83-38061cd6a8c8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24249,7 +24249,7 @@
           <xm:sqref>C24:O24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{a6de7bd0-e68f-4f22-9a4b-52508451c1bf}">
+          <x14:cfRule type="dataBar" id="{64fa7fee-d917-4de0-9f2c-445b0d3c0cea}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24262,7 +24262,7 @@
           <xm:sqref>C27:O27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2f855105-ca70-48e9-bb22-0a86855ee54f}">
+          <x14:cfRule type="dataBar" id="{599f4c3d-84b4-43cf-9e7e-b4e2885abd59}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24275,7 +24275,7 @@
           <xm:sqref>C36:O36</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{bbf82617-38a1-4e97-9e72-eb5a0c3bdb92}">
+          <x14:cfRule type="dataBar" id="{c327917d-ddae-4604-a315-4ee53f7f857f}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24288,7 +24288,7 @@
           <xm:sqref>C44:N44</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{60698893-4c65-4d50-af79-65729be2c6b5}">
+          <x14:cfRule type="dataBar" id="{278383ae-5d9e-4ba1-9eab-ce54cad1a3e3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24301,7 +24301,7 @@
           <xm:sqref>O44</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0d3ac796-bdc0-45d4-8882-852723bc1c17}">
+          <x14:cfRule type="dataBar" id="{d40bccc4-781f-478a-91c5-afe98f15aeaf}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24314,7 +24314,7 @@
           <xm:sqref>C52:N52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{261db87c-1e88-4ec8-bfd4-f9ff58e6ab69}">
+          <x14:cfRule type="dataBar" id="{e0e54f1a-610f-44d6-9a42-75de4393b59c}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24327,7 +24327,7 @@
           <xm:sqref>O52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{c7327550-3ab0-47f9-87ae-ebc7daa8c728}">
+          <x14:cfRule type="dataBar" id="{55f821aa-6302-4bc2-9058-472ebe7b94cd}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24340,7 +24340,7 @@
           <xm:sqref>C60:N60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{cd911691-1116-42fe-bc53-67b1c0267f3b}">
+          <x14:cfRule type="dataBar" id="{d3866566-82c4-41d8-a6c1-357419a7e181}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24353,7 +24353,7 @@
           <xm:sqref>O60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{488d3490-7eae-4875-a20c-b6e313a891f8}">
+          <x14:cfRule type="dataBar" id="{041a0567-316c-4c6c-b59c-04cc0a128409}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24366,7 +24366,7 @@
           <xm:sqref>C68:N68</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d32d3730-c799-495f-ab3f-368a55c0587b}">
+          <x14:cfRule type="dataBar" id="{13edfe20-6c42-4c8d-af9d-9e2ec69aeaae}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24379,7 +24379,7 @@
           <xm:sqref>O68</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{917a537d-9e87-4c62-970e-2a3208257cff}">
+          <x14:cfRule type="dataBar" id="{3145c08a-d8f1-4263-b847-f6ca27453b95}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24392,7 +24392,7 @@
           <xm:sqref>C76:N76</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{a0816f8a-cf6d-4ed6-be91-32fb8a7baa2b}">
+          <x14:cfRule type="dataBar" id="{cf2b4519-b2fb-4cc8-a377-bc0c000da78d}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24405,7 +24405,7 @@
           <xm:sqref>O76</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{46e4e21c-a7ec-4379-8b05-59f6f8733a0d}">
+          <x14:cfRule type="dataBar" id="{d54ffcba-f4e0-4a29-a988-b266d9749fea}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24418,7 +24418,7 @@
           <xm:sqref>C132:O132</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{62b58732-fa75-415f-ae8c-e06cbb39486c}">
+          <x14:cfRule type="dataBar" id="{135f8d21-d3d4-4de5-ae41-c1e1d6d183bb}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24431,7 +24431,7 @@
           <xm:sqref>C26:O26 D27:N27 C28:O28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{71e9fd37-0a20-44b6-bc97-8c3bc7b56d3c}">
+          <x14:cfRule type="dataBar" id="{7f5dccef-1bfb-492c-810e-be66cdfe0aaf}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24444,7 +24444,7 @@
           <xm:sqref>C35:O35 D36:N36 C37:O37</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1f554681-6d53-4dfd-9c51-909b0684a3a5}">
+          <x14:cfRule type="dataBar" id="{c23207e8-182b-40b1-9bcb-03876318e320}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24457,7 +24457,7 @@
           <xm:sqref>C43:N43 D44:N44 C45:N45</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{53a4cf40-caa0-4fba-a9ce-286287c1ff0d}">
+          <x14:cfRule type="dataBar" id="{aaac129a-cbca-490b-b1be-888331b9f70a}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24470,7 +24470,7 @@
           <xm:sqref>O43 O45</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7257bc84-0606-4596-9096-c367964143e1}">
+          <x14:cfRule type="dataBar" id="{c8cba163-b45a-4e26-a0ba-9a227b6f777a}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24483,7 +24483,7 @@
           <xm:sqref>C51:N51 D52:N52 C53:N53</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{b53cb82c-b426-442c-9227-d43032399732}">
+          <x14:cfRule type="dataBar" id="{d7451388-b77c-4e86-8099-85feb02bc130}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24496,7 +24496,7 @@
           <xm:sqref>O51 O53</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{b670fcd2-c030-4af4-a7c8-fa413a7d467a}">
+          <x14:cfRule type="dataBar" id="{f46ba46a-a72d-4c82-bc6b-466cc725a101}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24509,7 +24509,7 @@
           <xm:sqref>C59:N59 D60:N60 C61:N61</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3b8e60aa-309d-4e94-9e38-064c7c48539b}">
+          <x14:cfRule type="dataBar" id="{596bc0b3-802d-4592-94cc-81c20fd68aa5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24522,7 +24522,7 @@
           <xm:sqref>O59 O61</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8004c6e5-6aef-472d-9deb-d7bb3eb0a282}">
+          <x14:cfRule type="dataBar" id="{62f6e842-9461-4335-ab10-020b94a0c86c}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24535,7 +24535,7 @@
           <xm:sqref>C67:N67 D68:N68 C69:N69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8514cc6f-c463-4734-8c35-aebf1ed97435}">
+          <x14:cfRule type="dataBar" id="{333ac094-d46f-4ba5-aa34-e2c597442e72}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24548,7 +24548,7 @@
           <xm:sqref>O67 O69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{a79d2cca-63f7-4381-b276-ddc721ebedda}">
+          <x14:cfRule type="dataBar" id="{e00d3cdb-d6b7-493d-a01d-92157d3877d2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24561,7 +24561,7 @@
           <xm:sqref>C75:N75 D76:N76 C77:N77</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{830a7799-181e-4617-84cd-a83d5c0c5070}">
+          <x14:cfRule type="dataBar" id="{1efa4371-2280-4078-b7a9-4bed4b5c3ad8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24574,7 +24574,7 @@
           <xm:sqref>O75 O77</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d533caa9-ee38-4a38-89c9-b295f24de74e}">
+          <x14:cfRule type="dataBar" id="{afa2d65e-8b95-482b-9232-62e59aa41830}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24587,7 +24587,7 @@
           <xm:sqref>C83:N83 D84:N84 C85:O85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{af742c9d-636f-4fff-ac6a-7f9c7f3c7037}">
+          <x14:cfRule type="dataBar" id="{26e8731e-9f2a-41b7-b680-0ccbeee0b679}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24600,7 +24600,7 @@
           <xm:sqref>C84:O84 D85:N85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{81f1277b-500d-4e6c-aadd-268bf1ea342a}">
+          <x14:cfRule type="dataBar" id="{3cdc7788-f761-42e3-be98-2218d145b981}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24613,7 +24613,7 @@
           <xm:sqref>C91:N91 D92:N92 C93:O93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{e850438a-52e9-4882-a1ef-da02391dd87e}">
+          <x14:cfRule type="dataBar" id="{33a32dd6-7c3d-4131-bff3-5d7a133657f6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24626,7 +24626,7 @@
           <xm:sqref>C92:O92 D93:N93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3ac28c79-7159-43ed-93c3-5211aa02ceeb}">
+          <x14:cfRule type="dataBar" id="{57339abf-3c6b-4c81-a843-3b96853dd772}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24639,7 +24639,7 @@
           <xm:sqref>C99:N99 D100:N100 C101:O101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2e892bd2-e689-47f3-a102-223c279a2883}">
+          <x14:cfRule type="dataBar" id="{c5cc5271-65d0-4a0f-8cee-d2a5303bff74}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24652,7 +24652,7 @@
           <xm:sqref>C100:O100 D101:N101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{a7bf0662-6c40-4e21-832f-22511f489591}">
+          <x14:cfRule type="dataBar" id="{26477af8-b059-4a6c-965b-a6f139d7679b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24665,7 +24665,7 @@
           <xm:sqref>C107:N107 D108:N108 C109:O109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3baefdbb-4bb1-49bd-a3d7-cd63bcb4e76f}">
+          <x14:cfRule type="dataBar" id="{38415ac6-3eea-4117-b45e-fee9baecd296}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24678,7 +24678,7 @@
           <xm:sqref>C108:O108 D109:N109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{b197a809-348b-44d9-a999-27a78e001bfc}">
+          <x14:cfRule type="dataBar" id="{160e3e68-d9eb-41ff-a4b9-cf41893e7cd5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24691,7 +24691,7 @@
           <xm:sqref>C115:N115 D116:N116 C117:O117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{f4d769d6-5e2c-4223-8934-90e7dffbf419}">
+          <x14:cfRule type="dataBar" id="{cb18ce02-89e7-4e45-b6bf-6c71c8b5ffe8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24704,7 +24704,7 @@
           <xm:sqref>C116:O116 D117:N117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8c1fd285-8e9d-444b-a958-7c4598e8275c}">
+          <x14:cfRule type="dataBar" id="{904cf8e6-f644-4be8-b62c-6bc421b3bf03}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24717,7 +24717,7 @@
           <xm:sqref>C123:N123 D124:N124 C125:O125</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{622dc457-61a6-47ea-9505-488aaa864ee4}">
+          <x14:cfRule type="dataBar" id="{ec21f11a-afe1-4d6c-aac2-cdcf67fc6d02}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24730,7 +24730,7 @@
           <xm:sqref>C124:O124 D125:N125</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8e4e4590-eeec-47e3-a926-0c76b04861bd}">
+          <x14:cfRule type="dataBar" id="{2dae02d0-c2f2-4046-a497-b9cb14f37060}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26456,7 +26456,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{81f6f9e7-a985-4595-adcf-3a0b98bc49bb}</x14:id>
+          <x14:id>{fa99523b-e76c-456c-bd7e-f6bf2bea820e}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26470,7 +26470,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{492ab320-c910-4d9f-bb38-fa418698743b}</x14:id>
+          <x14:id>{6718fbf1-1f87-49f5-af7a-e3396e62aaf4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26484,7 +26484,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{23710130-a404-4e03-b99c-b36e79187513}</x14:id>
+          <x14:id>{643c1a5e-ce2e-4677-8a5c-580b25e329a1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26498,7 +26498,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{02654944-0412-40c4-a564-137086f6bf63}</x14:id>
+          <x14:id>{7a2bb73b-5023-4039-8a00-e55ff4db7eb4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26512,7 +26512,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7044294f-93cf-4e36-b9dc-7dab8caef34b}</x14:id>
+          <x14:id>{c44cdf66-e4f9-4634-acbc-89e31d062a8e}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26526,7 +26526,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{25ae9d96-b049-4461-b09c-042899fb4ac6}</x14:id>
+          <x14:id>{2a0942f2-e06a-47f9-b53c-ae88b526adb3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26540,7 +26540,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{adc8488e-6421-44dd-900c-9a23f9ff6039}</x14:id>
+          <x14:id>{c4c0aaec-eebf-46ce-9dba-765bccaaa73d}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26554,7 +26554,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0dcc808e-d7ee-4908-a9c0-8e203edd6295}</x14:id>
+          <x14:id>{b9f014e2-053c-4e4e-874c-02b5f83d3d2d}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26568,7 +26568,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0a36933a-2306-495d-8147-0d65717d43fc}</x14:id>
+          <x14:id>{f57805e7-f846-4c12-8bb3-3790f1ce9b59}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26582,7 +26582,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{b42e1ef0-8e80-4fa5-bbcd-0b27a29214dc}</x14:id>
+          <x14:id>{f6ebb3ee-83b4-42b6-8a06-840ce59b0814}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26596,7 +26596,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8cf0b732-c7ec-430c-b293-609a1988cd87}</x14:id>
+          <x14:id>{a8138153-7df2-4f57-8b52-72dd9039d758}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26632,7 +26632,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{51bd2f33-25b6-40c5-b8c2-bfdf71dada50}</x14:id>
+          <x14:id>{678360a4-2809-4c40-8343-58e66d1d4810}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26651,7 +26651,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{81f6f9e7-a985-4595-adcf-3a0b98bc49bb}">
+          <x14:cfRule type="dataBar" id="{fa99523b-e76c-456c-bd7e-f6bf2bea820e}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26664,7 +26664,7 @@
           <xm:sqref>C8:N8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{492ab320-c910-4d9f-bb38-fa418698743b}">
+          <x14:cfRule type="dataBar" id="{6718fbf1-1f87-49f5-af7a-e3396e62aaf4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26677,7 +26677,7 @@
           <xm:sqref>O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{23710130-a404-4e03-b99c-b36e79187513}">
+          <x14:cfRule type="dataBar" id="{643c1a5e-ce2e-4677-8a5c-580b25e329a1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26690,7 +26690,7 @@
           <xm:sqref>C12:N12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{02654944-0412-40c4-a564-137086f6bf63}">
+          <x14:cfRule type="dataBar" id="{7a2bb73b-5023-4039-8a00-e55ff4db7eb4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26703,7 +26703,7 @@
           <xm:sqref>O12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7044294f-93cf-4e36-b9dc-7dab8caef34b}">
+          <x14:cfRule type="dataBar" id="{c44cdf66-e4f9-4634-acbc-89e31d062a8e}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26716,7 +26716,7 @@
           <xm:sqref>C16:N16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{25ae9d96-b049-4461-b09c-042899fb4ac6}">
+          <x14:cfRule type="dataBar" id="{2a0942f2-e06a-47f9-b53c-ae88b526adb3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26729,7 +26729,7 @@
           <xm:sqref>O16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{adc8488e-6421-44dd-900c-9a23f9ff6039}">
+          <x14:cfRule type="dataBar" id="{c4c0aaec-eebf-46ce-9dba-765bccaaa73d}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26742,7 +26742,7 @@
           <xm:sqref>B20:N20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0dcc808e-d7ee-4908-a9c0-8e203edd6295}">
+          <x14:cfRule type="dataBar" id="{b9f014e2-053c-4e4e-874c-02b5f83d3d2d}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26755,7 +26755,7 @@
           <xm:sqref>O20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0a36933a-2306-495d-8147-0d65717d43fc}">
+          <x14:cfRule type="dataBar" id="{f57805e7-f846-4c12-8bb3-3790f1ce9b59}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26768,7 +26768,7 @@
           <xm:sqref>C24:N24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{b42e1ef0-8e80-4fa5-bbcd-0b27a29214dc}">
+          <x14:cfRule type="dataBar" id="{f6ebb3ee-83b4-42b6-8a06-840ce59b0814}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26781,7 +26781,7 @@
           <xm:sqref>O24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8cf0b732-c7ec-430c-b293-609a1988cd87}">
+          <x14:cfRule type="dataBar" id="{a8138153-7df2-4f57-8b52-72dd9039d758}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26794,7 +26794,7 @@
           <xm:sqref>C27:O27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{51bd2f33-25b6-40c5-b8c2-bfdf71dada50}">
+          <x14:cfRule type="dataBar" id="{678360a4-2809-4c40-8343-58e66d1d4810}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -37358,7 +37358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{95e38986-13f3-4134-a3ab-464e4333021e}</x14:id>
+          <x14:id>{9c5d1ad8-68f3-4434-87e3-5eddface94d6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37372,7 +37372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7f3d41e2-12d0-45e6-86ed-f2545223035e}</x14:id>
+          <x14:id>{ad83cb38-f319-4c0d-87c8-2258e6938332}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37386,7 +37386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{00786b7a-4d6e-4d72-9dbe-59bd2a9021b4}</x14:id>
+          <x14:id>{185753e8-8247-4775-a006-cd42020e4dd7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37400,7 +37400,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6a39f0f8-f35e-457c-8958-8bfc3188f406}</x14:id>
+          <x14:id>{e0ec31ee-bc8a-4163-995b-51fcfa9f8778}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37414,7 +37414,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{90fd3eeb-e676-46ed-85fe-cf5c569eaa07}</x14:id>
+          <x14:id>{2d4fe035-cc6f-4518-9be5-e680f27787db}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37428,7 +37428,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{f7e47fde-d34f-414a-bfad-fb93a8103ebe}</x14:id>
+          <x14:id>{0cb395b8-a082-432b-9367-16ae43cdd4cd}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37448,7 +37448,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{24fe019d-b07f-40bc-9318-ec76f69f46aa}</x14:id>
+          <x14:id>{279fc306-3f8f-4f23-bf93-70fe7f296f4b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37462,7 +37462,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{e9524932-71df-451c-b926-486c5988d721}</x14:id>
+          <x14:id>{8994d41d-2cca-42c8-b08f-b34a540185ce}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37476,7 +37476,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{69844d1e-6354-4ea9-a16a-393556ad8f3a}</x14:id>
+          <x14:id>{131e2ecd-b6e8-476b-b4f1-17c6f3b19401}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37490,7 +37490,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1709ccbb-d311-400f-8bb5-041aafdc79f4}</x14:id>
+          <x14:id>{38fb1d6d-f8fc-4dc7-b739-e19ec71b41fa}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37504,7 +37504,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{79c1445a-b224-49c9-ba7a-0bb7b9b59c55}</x14:id>
+          <x14:id>{650d4031-5e2c-4ee4-99ae-76f68ed1eb37}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37518,7 +37518,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9c6b8a00-7d4b-40a8-9f07-efc39709298b}</x14:id>
+          <x14:id>{ca5e0387-2f7a-4c75-89d8-612eab6b2034}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37540,7 +37540,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{310691b8-7273-4ed0-8e12-9c04b1858683}</x14:id>
+          <x14:id>{ae1b9f0c-36cf-42a9-b85a-d1b04b969df0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37570,7 +37570,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2dc7f2a3-79c9-4808-b398-f036df91731a}</x14:id>
+          <x14:id>{5bb72168-38cf-4dce-b191-e66c8bb4b785}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37600,7 +37600,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{bd1c12ce-95d1-40c1-aace-82fb4f7dc827}</x14:id>
+          <x14:id>{73a26aef-7573-4833-8201-ad23c9542779}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37630,7 +37630,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{20ddf07f-1c7d-4559-aee1-12a6acd8a38d}</x14:id>
+          <x14:id>{884886ec-50e5-4da8-b430-37e8bdc9cd33}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37660,7 +37660,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{cef98b52-0b11-4a9c-be4a-13d8a494f1ec}</x14:id>
+          <x14:id>{7052b3a1-c659-43e4-96c9-b89800d15fc2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37690,7 +37690,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{af839d7c-6ff7-4142-b5c4-f456c67d8099}</x14:id>
+          <x14:id>{30dfc89d-1a76-4549-918f-f1394c193faa}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37712,7 +37712,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{38536115-c2f8-4d86-821b-1abe20c40d3f}</x14:id>
+          <x14:id>{1936c832-5108-4be7-b2a5-651fa920cacd}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37734,7 +37734,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{823bf1f5-a28f-4a49-adce-836f776ab77d}</x14:id>
+          <x14:id>{bf863f1b-f2ea-4051-862a-f0361cc144e9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37756,7 +37756,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{90ba7c2d-555d-448d-9dbb-b05e7846ec6a}</x14:id>
+          <x14:id>{0f464481-e54c-43b3-81b3-3c90ac6017e8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37778,7 +37778,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0d7dc7b0-474a-48a0-bf05-c0231a534939}</x14:id>
+          <x14:id>{5ed325c7-2e03-4f7e-b6d3-76ee1bd3fbb7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37800,7 +37800,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{47249e09-f8e1-4d9c-93e6-fdde79d2c211}</x14:id>
+          <x14:id>{2515b826-6e0a-49c2-81d7-e1281ef64b1d}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37822,7 +37822,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{e3366ba3-8af1-44e9-9106-7dee791527fe}</x14:id>
+          <x14:id>{eae00273-fece-47e5-82a0-3fa174f3bf69}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37844,7 +37844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d43623ff-4657-4dfb-898b-d4a19feaabe2}</x14:id>
+          <x14:id>{7602e6e7-fdb1-49c7-861c-af5aeba6922c}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37866,7 +37866,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{bebaef2a-c51e-4ded-9698-10c8a071eb6a}</x14:id>
+          <x14:id>{265b9507-cdbd-4caf-8a3a-84ecbd8380bb}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37888,7 +37888,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{efd6c414-1292-4c0a-b55f-393891542356}</x14:id>
+          <x14:id>{cdd6ebab-35a8-4277-a4b2-dd4631c7352a}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37910,7 +37910,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ce0b600b-adea-430e-9ed1-63b72605c66a}</x14:id>
+          <x14:id>{4d04061a-c38b-464a-96a9-172a76c739ea}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37932,7 +37932,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{27ce5550-deec-41c4-8081-12e8ed33749b}</x14:id>
+          <x14:id>{ba0b1fea-17d7-4e97-99a0-8d8e67710f74}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37954,7 +37954,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{b0642fa0-f9b6-402f-9ee9-8b5059320514}</x14:id>
+          <x14:id>{912ceddb-1d3c-49c6-809d-d9fcae8e3a5c}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37976,7 +37976,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{dd59f914-9f20-40ff-bebb-dce958874ab8}</x14:id>
+          <x14:id>{60685b8d-a148-4ce5-b46e-533821d785d1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37998,7 +37998,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{94bb21f3-a44f-4fa6-b987-57118c6cb0b3}</x14:id>
+          <x14:id>{58d55f2e-8d26-49c5-b9c6-0252ed45f587}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38017,7 +38017,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{95e38986-13f3-4134-a3ab-464e4333021e}">
+          <x14:cfRule type="dataBar" id="{9c5d1ad8-68f3-4434-87e3-5eddface94d6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38030,7 +38030,7 @@
           <xm:sqref>C8:O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7f3d41e2-12d0-45e6-86ed-f2545223035e}">
+          <x14:cfRule type="dataBar" id="{ad83cb38-f319-4c0d-87c8-2258e6938332}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38043,7 +38043,7 @@
           <xm:sqref>C12:O12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{00786b7a-4d6e-4d72-9dbe-59bd2a9021b4}">
+          <x14:cfRule type="dataBar" id="{185753e8-8247-4775-a006-cd42020e4dd7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38056,7 +38056,7 @@
           <xm:sqref>C16:O16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6a39f0f8-f35e-457c-8958-8bfc3188f406}">
+          <x14:cfRule type="dataBar" id="{e0ec31ee-bc8a-4163-995b-51fcfa9f8778}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38069,7 +38069,7 @@
           <xm:sqref>C20:O20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{90fd3eeb-e676-46ed-85fe-cf5c569eaa07}">
+          <x14:cfRule type="dataBar" id="{2d4fe035-cc6f-4518-9be5-e680f27787db}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38082,7 +38082,7 @@
           <xm:sqref>C24:O24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{f7e47fde-d34f-414a-bfad-fb93a8103ebe}">
+          <x14:cfRule type="dataBar" id="{0cb395b8-a082-432b-9367-16ae43cdd4cd}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38095,7 +38095,7 @@
           <xm:sqref>O26</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{24fe019d-b07f-40bc-9318-ec76f69f46aa}">
+          <x14:cfRule type="dataBar" id="{279fc306-3f8f-4f23-bf93-70fe7f296f4b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38108,7 +38108,7 @@
           <xm:sqref>C27:O27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{e9524932-71df-451c-b926-486c5988d721}">
+          <x14:cfRule type="dataBar" id="{8994d41d-2cca-42c8-b08f-b34a540185ce}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38121,7 +38121,7 @@
           <xm:sqref>C36:O36</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{69844d1e-6354-4ea9-a16a-393556ad8f3a}">
+          <x14:cfRule type="dataBar" id="{131e2ecd-b6e8-476b-b4f1-17c6f3b19401}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38134,7 +38134,7 @@
           <xm:sqref>C44:O44</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1709ccbb-d311-400f-8bb5-041aafdc79f4}">
+          <x14:cfRule type="dataBar" id="{38fb1d6d-f8fc-4dc7-b739-e19ec71b41fa}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38147,7 +38147,7 @@
           <xm:sqref>C52:O52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{79c1445a-b224-49c9-ba7a-0bb7b9b59c55}">
+          <x14:cfRule type="dataBar" id="{650d4031-5e2c-4ee4-99ae-76f68ed1eb37}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38160,7 +38160,7 @@
           <xm:sqref>C60:O60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9c6b8a00-7d4b-40a8-9f07-efc39709298b}">
+          <x14:cfRule type="dataBar" id="{ca5e0387-2f7a-4c75-89d8-612eab6b2034}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38173,7 +38173,7 @@
           <xm:sqref>C124:O124</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{310691b8-7273-4ed0-8e12-9c04b1858683}">
+          <x14:cfRule type="dataBar" id="{ae1b9f0c-36cf-42a9-b85a-d1b04b969df0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38186,7 +38186,7 @@
           <xm:sqref>C26:N26 D27:N27 C28:O28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2dc7f2a3-79c9-4808-b398-f036df91731a}">
+          <x14:cfRule type="dataBar" id="{5bb72168-38cf-4dce-b191-e66c8bb4b785}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38199,7 +38199,7 @@
           <xm:sqref>C35:N35 D36:N36 C37:O37</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{bd1c12ce-95d1-40c1-aace-82fb4f7dc827}">
+          <x14:cfRule type="dataBar" id="{73a26aef-7573-4833-8201-ad23c9542779}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38212,7 +38212,7 @@
           <xm:sqref>C43:N43 D44:N44 C45:O45</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{20ddf07f-1c7d-4559-aee1-12a6acd8a38d}">
+          <x14:cfRule type="dataBar" id="{884886ec-50e5-4da8-b430-37e8bdc9cd33}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38225,7 +38225,7 @@
           <xm:sqref>C51:N51 D52:N52 C53:O53</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{cef98b52-0b11-4a9c-be4a-13d8a494f1ec}">
+          <x14:cfRule type="dataBar" id="{7052b3a1-c659-43e4-96c9-b89800d15fc2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38238,7 +38238,7 @@
           <xm:sqref>C59:N59 D60:N60 C61:O61</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{af839d7c-6ff7-4142-b5c4-f456c67d8099}">
+          <x14:cfRule type="dataBar" id="{30dfc89d-1a76-4549-918f-f1394c193faa}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38251,7 +38251,7 @@
           <xm:sqref>C67:N67 D68:N68 C69:O69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{38536115-c2f8-4d86-821b-1abe20c40d3f}">
+          <x14:cfRule type="dataBar" id="{1936c832-5108-4be7-b2a5-651fa920cacd}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38264,7 +38264,7 @@
           <xm:sqref>C68:O68 D69:N69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{823bf1f5-a28f-4a49-adce-836f776ab77d}">
+          <x14:cfRule type="dataBar" id="{bf863f1b-f2ea-4051-862a-f0361cc144e9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38277,7 +38277,7 @@
           <xm:sqref>C75:N75 D76:N76 C77:O77</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{90ba7c2d-555d-448d-9dbb-b05e7846ec6a}">
+          <x14:cfRule type="dataBar" id="{0f464481-e54c-43b3-81b3-3c90ac6017e8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38290,7 +38290,7 @@
           <xm:sqref>C76:O76 D77:N77</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0d7dc7b0-474a-48a0-bf05-c0231a534939}">
+          <x14:cfRule type="dataBar" id="{5ed325c7-2e03-4f7e-b6d3-76ee1bd3fbb7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38303,7 +38303,7 @@
           <xm:sqref>C83:N83 D84:N84 C85:O85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{47249e09-f8e1-4d9c-93e6-fdde79d2c211}">
+          <x14:cfRule type="dataBar" id="{2515b826-6e0a-49c2-81d7-e1281ef64b1d}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38316,7 +38316,7 @@
           <xm:sqref>C84:O84 D85:N85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{e3366ba3-8af1-44e9-9106-7dee791527fe}">
+          <x14:cfRule type="dataBar" id="{eae00273-fece-47e5-82a0-3fa174f3bf69}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38329,7 +38329,7 @@
           <xm:sqref>C91:N91 D92:N92 C93:O93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d43623ff-4657-4dfb-898b-d4a19feaabe2}">
+          <x14:cfRule type="dataBar" id="{7602e6e7-fdb1-49c7-861c-af5aeba6922c}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38342,7 +38342,7 @@
           <xm:sqref>C92:O92 D93:N93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{bebaef2a-c51e-4ded-9698-10c8a071eb6a}">
+          <x14:cfRule type="dataBar" id="{265b9507-cdbd-4caf-8a3a-84ecbd8380bb}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38355,7 +38355,7 @@
           <xm:sqref>C99:N99 D100:N100 C101:O101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{efd6c414-1292-4c0a-b55f-393891542356}">
+          <x14:cfRule type="dataBar" id="{cdd6ebab-35a8-4277-a4b2-dd4631c7352a}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38368,7 +38368,7 @@
           <xm:sqref>C100:O100 D101:N101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ce0b600b-adea-430e-9ed1-63b72605c66a}">
+          <x14:cfRule type="dataBar" id="{4d04061a-c38b-464a-96a9-172a76c739ea}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38381,7 +38381,7 @@
           <xm:sqref>C107:N107 D108:N108 C109:O109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{27ce5550-deec-41c4-8081-12e8ed33749b}">
+          <x14:cfRule type="dataBar" id="{ba0b1fea-17d7-4e97-99a0-8d8e67710f74}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38394,7 +38394,7 @@
           <xm:sqref>C108:O108 D109:N109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{b0642fa0-f9b6-402f-9ee9-8b5059320514}">
+          <x14:cfRule type="dataBar" id="{912ceddb-1d3c-49c6-809d-d9fcae8e3a5c}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38407,7 +38407,7 @@
           <xm:sqref>C115:N115 D116:N116 C117:O117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{dd59f914-9f20-40ff-bebb-dce958874ab8}">
+          <x14:cfRule type="dataBar" id="{60685b8d-a148-4ce5-b46e-533821d785d1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38420,7 +38420,7 @@
           <xm:sqref>C116:O116 D117:N117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{94bb21f3-a44f-4fa6-b987-57118c6cb0b3}">
+          <x14:cfRule type="dataBar" id="{58d55f2e-8d26-49c5-b9c6-0252ed45f587}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -39902,7 +39902,7 @@
         <f>[3]陈欣诺!M8</f>
         <v>5719.5</v>
       </c>
-      <c r="O14" s="30">
+      <c r="O14" s="36">
         <f>SUM(C14:N14)</f>
         <v>80239.99</v>
       </c>
@@ -45989,7 +45989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4052ffb9-5868-461f-be15-eaca23cb5b83}</x14:id>
+          <x14:id>{fd07eebf-ad57-463d-99c1-fd3ec75ea292}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46003,7 +46003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{cf55cac8-7e19-4756-9971-340a54ac09ee}</x14:id>
+          <x14:id>{343f6457-bcab-4383-9b99-dd3497f6f19f}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46017,7 +46017,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{46505f3d-599d-46c0-8a12-9381d6ffd955}</x14:id>
+          <x14:id>{9fa8764b-6382-41d8-a03e-47733984e783}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46031,7 +46031,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{cbb022a6-4f86-435d-81f5-f191c1cc7fdf}</x14:id>
+          <x14:id>{8e4b3483-6a54-4439-aa00-6c5f95c3fdbd}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46045,7 +46045,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{552b9c34-e590-43cd-bc28-cbf71ad2b4d3}</x14:id>
+          <x14:id>{221221cf-574c-4b8b-aa5e-135f4187c80f}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46059,7 +46059,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{f4abbeed-8ed2-4133-90ea-73fd66af5c71}</x14:id>
+          <x14:id>{130ba751-1c36-4ba7-9e5a-3a1da5a2e1ae}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46073,7 +46073,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{c1c4381f-92a4-45c4-96ce-94ad69456211}</x14:id>
+          <x14:id>{0e5d675c-9da6-4078-a1ba-a1f4e2c3b183}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46087,7 +46087,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6356fa9c-67a8-4f0f-917d-53bb4ff4e43d}</x14:id>
+          <x14:id>{eaf9691d-e9c3-4d1f-a6f1-461b59983a0a}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46101,7 +46101,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1550b14f-5b10-405a-b3db-c8a18a1f94d6}</x14:id>
+          <x14:id>{2dcde596-dab4-4f85-910b-c8f6cfbfe036}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46115,7 +46115,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1926dcf0-7490-4ccd-a4f1-68c62ec183b1}</x14:id>
+          <x14:id>{9988af99-e592-42c7-8174-6070554d345b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46129,7 +46129,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{e8f6b5a1-80ba-4292-83aa-8cb0c7cf6c1c}</x14:id>
+          <x14:id>{9e4caeba-769d-4d44-8f63-1db346cfc980}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46165,7 +46165,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7a3a96a8-7a69-49ec-967d-78d7bde2f219}</x14:id>
+          <x14:id>{1ae04b52-5fb8-4270-9dcd-b6e0211ab32a}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46184,7 +46184,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4052ffb9-5868-461f-be15-eaca23cb5b83}">
+          <x14:cfRule type="dataBar" id="{fd07eebf-ad57-463d-99c1-fd3ec75ea292}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46197,7 +46197,7 @@
           <xm:sqref>C8:N8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{cf55cac8-7e19-4756-9971-340a54ac09ee}">
+          <x14:cfRule type="dataBar" id="{343f6457-bcab-4383-9b99-dd3497f6f19f}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46210,7 +46210,7 @@
           <xm:sqref>O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{46505f3d-599d-46c0-8a12-9381d6ffd955}">
+          <x14:cfRule type="dataBar" id="{9fa8764b-6382-41d8-a03e-47733984e783}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46223,7 +46223,7 @@
           <xm:sqref>C12:N12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{cbb022a6-4f86-435d-81f5-f191c1cc7fdf}">
+          <x14:cfRule type="dataBar" id="{8e4b3483-6a54-4439-aa00-6c5f95c3fdbd}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46236,7 +46236,7 @@
           <xm:sqref>O12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{552b9c34-e590-43cd-bc28-cbf71ad2b4d3}">
+          <x14:cfRule type="dataBar" id="{221221cf-574c-4b8b-aa5e-135f4187c80f}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46249,7 +46249,7 @@
           <xm:sqref>C16:N16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{f4abbeed-8ed2-4133-90ea-73fd66af5c71}">
+          <x14:cfRule type="dataBar" id="{130ba751-1c36-4ba7-9e5a-3a1da5a2e1ae}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46262,7 +46262,7 @@
           <xm:sqref>O16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{c1c4381f-92a4-45c4-96ce-94ad69456211}">
+          <x14:cfRule type="dataBar" id="{0e5d675c-9da6-4078-a1ba-a1f4e2c3b183}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46275,7 +46275,7 @@
           <xm:sqref>B20:N20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6356fa9c-67a8-4f0f-917d-53bb4ff4e43d}">
+          <x14:cfRule type="dataBar" id="{eaf9691d-e9c3-4d1f-a6f1-461b59983a0a}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46288,7 +46288,7 @@
           <xm:sqref>O20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1550b14f-5b10-405a-b3db-c8a18a1f94d6}">
+          <x14:cfRule type="dataBar" id="{2dcde596-dab4-4f85-910b-c8f6cfbfe036}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46301,7 +46301,7 @@
           <xm:sqref>C24:N24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1926dcf0-7490-4ccd-a4f1-68c62ec183b1}">
+          <x14:cfRule type="dataBar" id="{9988af99-e592-42c7-8174-6070554d345b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46314,7 +46314,7 @@
           <xm:sqref>O24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{e8f6b5a1-80ba-4292-83aa-8cb0c7cf6c1c}">
+          <x14:cfRule type="dataBar" id="{9e4caeba-769d-4d44-8f63-1db346cfc980}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46327,7 +46327,7 @@
           <xm:sqref>C27:O27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7a3a96a8-7a69-49ec-967d-78d7bde2f219}">
+          <x14:cfRule type="dataBar" id="{1ae04b52-5fb8-4270-9dcd-b6e0211ab32a}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
update weekly report data ver=202608261607
</commit_message>
<xml_diff>
--- a/2026WB年规进度.xlsx
+++ b/2026WB年规进度.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="13380" activeTab="4"/>
+    <workbookView windowWidth="29868" windowHeight="13380" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="毛立新" sheetId="1" r:id="rId1"/>
@@ -6531,6 +6531,8 @@
       <sheetName val="周度汇总分析报告"/>
       <sheetName val="2026年度男装数据汇总分析--俄罗斯"/>
       <sheetName val="2026年月度数据汇总--俄罗斯"/>
+      <sheetName val="2026年月度数据汇总-何欢洁"/>
+      <sheetName val="2026年月度数据汇总-郑志远"/>
       <sheetName val="2026年数据登记--俄罗斯"/>
       <sheetName val="2026目标拆解--俄罗斯"/>
       <sheetName val="2026目标拆解--俄罗斯 --实时调整"/>
@@ -6697,7 +6699,7 @@
             <v>593421.46</v>
           </cell>
           <cell r="H7">
-            <v>325038.63</v>
+            <v>637416.38</v>
           </cell>
           <cell r="I7">
             <v>0</v>
@@ -6718,7 +6720,7 @@
             <v>0</v>
           </cell>
           <cell r="O7">
-            <v>3437257.96</v>
+            <v>3749635.71</v>
           </cell>
         </row>
         <row r="8">
@@ -6741,7 +6743,7 @@
             <v>1.09246608580648</v>
           </cell>
           <cell r="H8">
-            <v>0.535748473942456</v>
+            <v>1.05062851406593</v>
           </cell>
           <cell r="I8">
             <v>0</v>
@@ -6762,7 +6764,7 @@
             <v>0</v>
           </cell>
           <cell r="O8">
-            <v>0.392593009981998</v>
+            <v>0.428271833786046</v>
           </cell>
         </row>
         <row r="10">
@@ -6829,7 +6831,7 @@
             <v>26753</v>
           </cell>
           <cell r="H11">
-            <v>15887</v>
+            <v>32761</v>
           </cell>
           <cell r="I11">
             <v>0</v>
@@ -6850,7 +6852,7 @@
             <v>0</v>
           </cell>
           <cell r="O11">
-            <v>171643</v>
+            <v>188517</v>
           </cell>
         </row>
         <row r="12">
@@ -6873,7 +6875,7 @@
             <v>0.743138888888889</v>
           </cell>
           <cell r="H12">
-            <v>0.395130201208745</v>
+            <v>0.814808366702315</v>
           </cell>
           <cell r="I12">
             <v>0</v>
@@ -6894,7 +6896,7 @@
             <v>0</v>
           </cell>
           <cell r="O12">
-            <v>0.295491950033742</v>
+            <v>0.324541379167872</v>
           </cell>
         </row>
         <row r="14">
@@ -6961,7 +6963,7 @@
             <v>9282</v>
           </cell>
           <cell r="H15">
-            <v>5500</v>
+            <v>11458</v>
           </cell>
           <cell r="I15">
             <v>0</v>
@@ -6982,7 +6984,7 @@
             <v>0</v>
           </cell>
           <cell r="O15">
-            <v>60846</v>
+            <v>66804</v>
           </cell>
         </row>
         <row r="16">
@@ -7005,7 +7007,7 @@
             <v>0.831720430107527</v>
           </cell>
           <cell r="H16">
-            <v>0.441264841541795</v>
+            <v>0.919275009888344</v>
           </cell>
           <cell r="I16">
             <v>0</v>
@@ -7026,7 +7028,7 @@
             <v>0</v>
           </cell>
           <cell r="O16">
-            <v>0.337901326548428</v>
+            <v>0.370988400531526</v>
           </cell>
         </row>
         <row r="18">
@@ -7093,7 +7095,7 @@
             <v>11545368.1632</v>
           </cell>
           <cell r="H19">
-            <v>6659288.4732</v>
+            <v>15086133.2796</v>
           </cell>
           <cell r="I19">
             <v>0</v>
@@ -7114,7 +7116,7 @@
             <v>0</v>
           </cell>
           <cell r="O19">
-            <v>67577309.1834</v>
+            <v>76004153.9898</v>
           </cell>
         </row>
         <row r="20">
@@ -7137,7 +7139,7 @@
             <v>0.922448718696069</v>
           </cell>
           <cell r="H20">
-            <v>0.476369032961964</v>
+            <v>1.07917936735439</v>
           </cell>
           <cell r="I20">
             <v>0</v>
@@ -7158,7 +7160,7 @@
             <v>0</v>
           </cell>
           <cell r="O20">
-            <v>0.335043434341862</v>
+            <v>0.376823124280976</v>
           </cell>
         </row>
         <row r="22">
@@ -7225,7 +7227,7 @@
             <v>3503371.5464</v>
           </cell>
           <cell r="H23">
-            <v>1930982.2827</v>
+            <v>4076553.6474</v>
           </cell>
           <cell r="I23">
             <v>0</v>
@@ -7246,7 +7248,7 @@
             <v>0</v>
           </cell>
           <cell r="O23">
-            <v>21876883.9391</v>
+            <v>24022455.3038</v>
           </cell>
         </row>
         <row r="24">
@@ -7269,7 +7271,7 @@
             <v>0.874723240851709</v>
           </cell>
           <cell r="H24">
-            <v>0.431662184320827</v>
+            <v>0.911294768317202</v>
           </cell>
           <cell r="I24">
             <v>0</v>
@@ -7290,7 +7292,7 @@
             <v>0</v>
           </cell>
           <cell r="O24">
-            <v>0.33895004922076</v>
+            <v>0.372192512895943</v>
           </cell>
         </row>
         <row r="26">
@@ -7313,7 +7315,7 @@
             <v>0.30344390034843</v>
           </cell>
           <cell r="H26">
-            <v>0.289968258691773</v>
+            <v>0.270218588941704</v>
           </cell>
           <cell r="I26" t="e">
             <v>#DIV/0!</v>
@@ -7334,7 +7336,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O26">
-            <v>0.323731208055765</v>
+            <v>0.316067662657279</v>
           </cell>
         </row>
         <row r="27">
@@ -7357,7 +7359,7 @@
             <v>0.653048256270325</v>
           </cell>
           <cell r="H27">
-            <v>0.653804997796941</v>
+            <v>0.65025487622478</v>
           </cell>
           <cell r="I27" t="e">
             <v>#DIV/0!</v>
@@ -7378,7 +7380,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O27">
-            <v>0.645508409897287</v>
+            <v>0.645634080746033</v>
           </cell>
         </row>
         <row r="28">
@@ -7401,7 +7403,7 @@
             <v>0.16938581938584</v>
           </cell>
           <cell r="H28">
-            <v>0.168328126525073</v>
+            <v>0.156361582634032</v>
           </cell>
           <cell r="I28" t="e">
             <v>#DIV/0!</v>
@@ -7422,7 +7424,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O28">
-            <v>0.157118260972107</v>
+            <v>0.156088778710595</v>
           </cell>
         </row>
         <row r="30">
@@ -7448,7 +7450,7 @@
             <v>213687.24</v>
           </cell>
           <cell r="H30">
-            <v>102754.41</v>
+            <v>196174.75</v>
           </cell>
           <cell r="I30">
             <v>0</v>
@@ -7469,7 +7471,7 @@
             <v>0</v>
           </cell>
           <cell r="O30">
-            <v>1874915.07</v>
+            <v>1968335.41</v>
           </cell>
         </row>
         <row r="31">
@@ -7492,7 +7494,7 @@
             <v>10453</v>
           </cell>
           <cell r="H31">
-            <v>5785</v>
+            <v>11621</v>
           </cell>
           <cell r="I31">
             <v>0</v>
@@ -7513,7 +7515,7 @@
             <v>0</v>
           </cell>
           <cell r="O31">
-            <v>82089</v>
+            <v>87925</v>
           </cell>
         </row>
         <row r="32">
@@ -7536,7 +7538,7 @@
             <v>3602</v>
           </cell>
           <cell r="H32">
-            <v>1927</v>
+            <v>3917</v>
           </cell>
           <cell r="I32">
             <v>0</v>
@@ -7557,7 +7559,7 @@
             <v>0</v>
           </cell>
           <cell r="O32">
-            <v>30081</v>
+            <v>32071</v>
           </cell>
         </row>
         <row r="33">
@@ -7580,7 +7582,7 @@
             <v>4439731.0488</v>
           </cell>
           <cell r="H33">
-            <v>2511111.222</v>
+            <v>5199070.2324</v>
           </cell>
           <cell r="I33">
             <v>0</v>
@@ -7601,7 +7603,7 @@
             <v>0</v>
           </cell>
           <cell r="O33">
-            <v>33826837.7889</v>
+            <v>36514796.7993</v>
           </cell>
         </row>
         <row r="34">
@@ -7624,7 +7626,7 @@
             <v>1407371.462</v>
           </cell>
           <cell r="H34">
-            <v>699411.4057</v>
+            <v>1456186.0782</v>
           </cell>
           <cell r="I34">
             <v>0</v>
@@ -7645,7 +7647,7 @@
             <v>0</v>
           </cell>
           <cell r="O34">
-            <v>11088070.4977</v>
+            <v>11844845.1702</v>
           </cell>
         </row>
         <row r="35">
@@ -7668,7 +7670,7 @@
             <v>0.316994756333358</v>
           </cell>
           <cell r="H35">
-            <v>0.278526653687186</v>
+            <v>0.280085864031076</v>
           </cell>
           <cell r="I35" t="e">
             <v>#DIV/0!</v>
@@ -7689,7 +7691,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O35">
-            <v>0.327789152710528</v>
+            <v>0.324384803106095</v>
           </cell>
         </row>
         <row r="36">
@@ -7712,7 +7714,7 @@
             <v>0.655409930163589</v>
           </cell>
           <cell r="H36">
-            <v>0.666897147796024</v>
+            <v>0.662937785044316</v>
           </cell>
           <cell r="I36" t="e">
             <v>#DIV/0!</v>
@@ -7733,7 +7735,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O36">
-            <v>0.633556262105763</v>
+            <v>0.635245948251351</v>
           </cell>
         </row>
         <row r="37">
@@ -7756,7 +7758,7 @@
             <v>0.15183428524004</v>
           </cell>
           <cell r="H37">
-            <v>0.1469155480774</v>
+            <v>0.134718188105804</v>
           </cell>
           <cell r="I37" t="e">
             <v>#DIV/0!</v>
@@ -7777,7 +7779,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O37">
-            <v>0.169092996873434</v>
+            <v>0.166176541923238</v>
           </cell>
         </row>
         <row r="38">
@@ -7803,7 +7805,7 @@
             <v>95805.82</v>
           </cell>
           <cell r="H38">
-            <v>77964.2</v>
+            <v>169438.85</v>
           </cell>
           <cell r="I38">
             <v>0</v>
@@ -7824,7 +7826,7 @@
             <v>0</v>
           </cell>
           <cell r="O38">
-            <v>651335.88</v>
+            <v>742810.53</v>
           </cell>
         </row>
         <row r="39">
@@ -7847,7 +7849,7 @@
             <v>6417</v>
           </cell>
           <cell r="H39">
-            <v>4008</v>
+            <v>9124</v>
           </cell>
           <cell r="I39">
             <v>0</v>
@@ -7868,7 +7870,7 @@
             <v>0</v>
           </cell>
           <cell r="O39">
-            <v>38083</v>
+            <v>43199</v>
           </cell>
         </row>
         <row r="40">
@@ -7891,7 +7893,7 @@
             <v>1916</v>
           </cell>
           <cell r="H40">
-            <v>1324</v>
+            <v>2945</v>
           </cell>
           <cell r="I40">
             <v>0</v>
@@ -7912,7 +7914,7 @@
             <v>0</v>
           </cell>
           <cell r="O40">
-            <v>12514</v>
+            <v>14135</v>
           </cell>
         </row>
         <row r="41">
@@ -7935,7 +7937,7 @@
             <v>2954093.3256</v>
           </cell>
           <cell r="H41">
-            <v>1634730.252</v>
+            <v>3813426.3168</v>
           </cell>
           <cell r="I41">
             <v>0</v>
@@ -7956,7 +7958,7 @@
             <v>0</v>
           </cell>
           <cell r="O41">
-            <v>14329032.7986</v>
+            <v>16507728.8634</v>
           </cell>
         </row>
         <row r="42">
@@ -7979,7 +7981,7 @@
             <v>702420.3795</v>
           </cell>
           <cell r="H42">
-            <v>458423.5943</v>
+            <v>1032316.5394</v>
           </cell>
           <cell r="I42">
             <v>0</v>
@@ -8000,7 +8002,7 @@
             <v>0</v>
           </cell>
           <cell r="O42">
-            <v>4184008.9538</v>
+            <v>4757901.8989</v>
           </cell>
         </row>
         <row r="43">
@@ -8023,7 +8025,7 @@
             <v>0.237778669147947</v>
           </cell>
           <cell r="H43">
-            <v>0.280427669176089</v>
+            <v>0.270705778384164</v>
           </cell>
           <cell r="I43" t="e">
             <v>#DIV/0!</v>
@@ -8044,7 +8046,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O43">
-            <v>0.291995210884631</v>
+            <v>0.288222682736748</v>
           </cell>
         </row>
         <row r="44">
@@ -8067,7 +8069,7 @@
             <v>0.701418108150226</v>
           </cell>
           <cell r="H44">
-            <v>0.669660678642715</v>
+            <v>0.677224901359053</v>
           </cell>
           <cell r="I44" t="e">
             <v>#DIV/0!</v>
@@ -8088,7 +8090,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O44">
-            <v>0.671401937872542</v>
+            <v>0.672793351697956</v>
           </cell>
         </row>
         <row r="45">
@@ -8111,7 +8113,7 @@
             <v>0.136393850173022</v>
           </cell>
           <cell r="H45">
-            <v>0.170070216649841</v>
+            <v>0.164134588116239</v>
           </cell>
           <cell r="I45" t="e">
             <v>#DIV/0!</v>
@@ -8132,7 +8134,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O45">
-            <v>0.155672678331255</v>
+            <v>0.156121447180686</v>
           </cell>
         </row>
         <row r="46">
@@ -8158,7 +8160,7 @@
             <v>267227.4</v>
           </cell>
           <cell r="H46">
-            <v>131378.65</v>
+            <v>246129.6</v>
           </cell>
           <cell r="I46">
             <v>0</v>
@@ -8179,7 +8181,7 @@
             <v>0</v>
           </cell>
           <cell r="O46">
-            <v>764491.77</v>
+            <v>879242.72</v>
           </cell>
         </row>
         <row r="47">
@@ -8202,7 +8204,7 @@
             <v>8516</v>
           </cell>
           <cell r="H47">
-            <v>5471</v>
+            <v>10835</v>
           </cell>
           <cell r="I47">
             <v>0</v>
@@ -8223,7 +8225,7 @@
             <v>0</v>
           </cell>
           <cell r="O47">
-            <v>34272</v>
+            <v>39636</v>
           </cell>
         </row>
         <row r="48">
@@ -8246,7 +8248,7 @@
             <v>3226</v>
           </cell>
           <cell r="H48">
-            <v>1994</v>
+            <v>4088</v>
           </cell>
           <cell r="I48">
             <v>0</v>
@@ -8267,7 +8269,7 @@
             <v>0</v>
           </cell>
           <cell r="O48">
-            <v>11970</v>
+            <v>14064</v>
           </cell>
         </row>
         <row r="49">
@@ -8290,7 +8292,7 @@
             <v>3625780.1448</v>
           </cell>
           <cell r="H49">
-            <v>2274149.9952</v>
+            <v>4595999.0844</v>
           </cell>
           <cell r="I49">
             <v>0</v>
@@ -8311,7 +8313,7 @@
             <v>0</v>
           </cell>
           <cell r="O49">
-            <v>13376634.4806</v>
+            <v>15698483.5698</v>
           </cell>
         </row>
         <row r="50">
@@ -8334,7 +8336,7 @@
             <v>1213786.7552</v>
           </cell>
           <cell r="H50">
-            <v>692555.2367</v>
+            <v>1427835.2688</v>
           </cell>
           <cell r="I50">
             <v>0</v>
@@ -8355,7 +8357,7 @@
             <v>0</v>
           </cell>
           <cell r="O50">
-            <v>4218986.3419</v>
+            <v>4954266.374</v>
           </cell>
         </row>
         <row r="51">
@@ -8378,7 +8380,7 @@
             <v>0.334765679860865</v>
           </cell>
           <cell r="H51">
-            <v>0.304533666715811</v>
+            <v>0.310669180428351</v>
           </cell>
           <cell r="I51" t="e">
             <v>#DIV/0!</v>
@@ -8399,7 +8401,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O51">
-            <v>0.315399688017098</v>
+            <v>0.315588849838387</v>
           </cell>
         </row>
         <row r="52">
@@ -8422,7 +8424,7 @@
             <v>0.621183654297792</v>
           </cell>
           <cell r="H52">
-            <v>0.635532809358435</v>
+            <v>0.622704199353945</v>
           </cell>
           <cell r="I52" t="e">
             <v>#DIV/0!</v>
@@ -8443,7 +8445,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O52">
-            <v>0.650735294117647</v>
+            <v>0.645171056615198</v>
           </cell>
         </row>
         <row r="53">
@@ -8466,7 +8468,7 @@
             <v>0.22016008895728</v>
           </cell>
           <cell r="H53">
-            <v>0.189701330721307</v>
+            <v>0.172379549222688</v>
           </cell>
           <cell r="I53" t="e">
             <v>#DIV/0!</v>
@@ -8487,7 +8489,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O53">
-            <v>0.181202712700823</v>
+            <v>0.177471830060303</v>
           </cell>
         </row>
         <row r="54">
@@ -8513,7 +8515,7 @@
             <v>16701</v>
           </cell>
           <cell r="H54">
-            <v>12941.37</v>
+            <v>25673.18</v>
           </cell>
           <cell r="I54">
             <v>0</v>
@@ -8534,7 +8536,7 @@
             <v>0</v>
           </cell>
           <cell r="O54">
-            <v>146515.24</v>
+            <v>159247.05</v>
           </cell>
         </row>
         <row r="55">
@@ -8557,7 +8559,7 @@
             <v>1367</v>
           </cell>
           <cell r="H55">
-            <v>623</v>
+            <v>1181</v>
           </cell>
           <cell r="I55">
             <v>0</v>
@@ -8578,7 +8580,7 @@
             <v>0</v>
           </cell>
           <cell r="O55">
-            <v>17199</v>
+            <v>17757</v>
           </cell>
         </row>
         <row r="56">
@@ -8601,7 +8603,7 @@
             <v>538</v>
           </cell>
           <cell r="H56">
-            <v>255</v>
+            <v>508</v>
           </cell>
           <cell r="I56">
             <v>0</v>
@@ -8622,7 +8624,7 @@
             <v>0</v>
           </cell>
           <cell r="O56">
-            <v>6281</v>
+            <v>6534</v>
           </cell>
         </row>
         <row r="57">
@@ -8645,7 +8647,7 @@
             <v>525763.644</v>
           </cell>
           <cell r="H57">
-            <v>239297.004</v>
+            <v>1477637.646</v>
           </cell>
           <cell r="I57">
             <v>0</v>
@@ -8666,7 +8668,7 @@
             <v>0</v>
           </cell>
           <cell r="O57">
-            <v>6044804.1153</v>
+            <v>7283144.7573</v>
           </cell>
         </row>
         <row r="58">
@@ -8689,7 +8691,7 @@
             <v>179792.9497</v>
           </cell>
           <cell r="H58">
-            <v>80592.046</v>
+            <v>160215.761</v>
           </cell>
           <cell r="I58">
             <v>0</v>
@@ -8710,7 +8712,7 @@
             <v>0</v>
           </cell>
           <cell r="O58">
-            <v>2385818.1457</v>
+            <v>2465441.8607</v>
           </cell>
         </row>
         <row r="59">
@@ -8733,7 +8735,7 @@
             <v>0.341965352210622</v>
           </cell>
           <cell r="H59">
-            <v>0.336786690400854</v>
+            <v>0.108426962072676</v>
           </cell>
           <cell r="I59" t="e">
             <v>#DIV/0!</v>
@@ -8754,7 +8756,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O59">
-            <v>0.394689075144926</v>
+            <v>0.338513367900432</v>
           </cell>
         </row>
         <row r="60">
@@ -8777,7 +8779,7 @@
             <v>0.606437454279444</v>
           </cell>
           <cell r="H60">
-            <v>0.590690208667737</v>
+            <v>0.569856054191363</v>
           </cell>
           <cell r="I60" t="e">
             <v>#DIV/0!</v>
@@ -8798,7 +8800,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O60">
-            <v>0.634804349090063</v>
+            <v>0.632032437911809</v>
           </cell>
         </row>
         <row r="61">
@@ -8821,7 +8823,7 @@
             <v>0.0928901830014306</v>
           </cell>
           <cell r="H61">
-            <v>0.160578749917827</v>
+            <v>0.160241288620787</v>
           </cell>
           <cell r="I61" t="e">
             <v>#DIV/0!</v>
@@ -8842,7 +8844,7 @@
             <v>#DIV/0!</v>
           </cell>
           <cell r="O61">
-            <v>0.0614109001828437</v>
+            <v>0.0645916874124891</v>
           </cell>
         </row>
         <row r="62">
@@ -11704,7 +11706,7 @@
             <v>213687.24</v>
           </cell>
           <cell r="H3">
-            <v>102754.41</v>
+            <v>196174.75</v>
           </cell>
           <cell r="I3">
             <v>0</v>
@@ -11742,7 +11744,7 @@
             <v>10453</v>
           </cell>
           <cell r="H4">
-            <v>5785</v>
+            <v>11621</v>
           </cell>
           <cell r="I4">
             <v>0</v>
@@ -11780,7 +11782,7 @@
             <v>3602</v>
           </cell>
           <cell r="H5">
-            <v>1927</v>
+            <v>3917</v>
           </cell>
           <cell r="I5">
             <v>0</v>
@@ -11818,7 +11820,7 @@
             <v>4439731.0488</v>
           </cell>
           <cell r="H6">
-            <v>2511111.222</v>
+            <v>5199070.2324</v>
           </cell>
           <cell r="I6">
             <v>0</v>
@@ -11856,7 +11858,7 @@
             <v>95805.82</v>
           </cell>
           <cell r="H8">
-            <v>77964.2</v>
+            <v>169438.85</v>
           </cell>
           <cell r="I8">
             <v>0</v>
@@ -11894,7 +11896,7 @@
             <v>6417</v>
           </cell>
           <cell r="H9">
-            <v>4008</v>
+            <v>9124</v>
           </cell>
           <cell r="I9">
             <v>0</v>
@@ -11932,7 +11934,7 @@
             <v>1916</v>
           </cell>
           <cell r="H10">
-            <v>1324</v>
+            <v>2945</v>
           </cell>
           <cell r="I10">
             <v>0</v>
@@ -11970,7 +11972,7 @@
             <v>2954093.3256</v>
           </cell>
           <cell r="H11">
-            <v>1634730.252</v>
+            <v>3813426.3168</v>
           </cell>
           <cell r="I11">
             <v>0</v>
@@ -12008,7 +12010,7 @@
             <v>267227.4</v>
           </cell>
           <cell r="H13">
-            <v>131378.65</v>
+            <v>246129.6</v>
           </cell>
           <cell r="I13">
             <v>0</v>
@@ -12046,7 +12048,7 @@
             <v>8516</v>
           </cell>
           <cell r="H14">
-            <v>5471</v>
+            <v>10835</v>
           </cell>
           <cell r="I14">
             <v>0</v>
@@ -12084,7 +12086,7 @@
             <v>3226</v>
           </cell>
           <cell r="H15">
-            <v>1994</v>
+            <v>4088</v>
           </cell>
           <cell r="I15">
             <v>0</v>
@@ -12122,7 +12124,7 @@
             <v>3625780.1448</v>
           </cell>
           <cell r="H16">
-            <v>2274149.9952</v>
+            <v>4595999.0844</v>
           </cell>
           <cell r="I16">
             <v>0</v>
@@ -12160,7 +12162,7 @@
             <v>16701</v>
           </cell>
           <cell r="H18">
-            <v>12941.37</v>
+            <v>25673.18</v>
           </cell>
           <cell r="I18">
             <v>0</v>
@@ -12198,7 +12200,7 @@
             <v>1367</v>
           </cell>
           <cell r="H19">
-            <v>623</v>
+            <v>1181</v>
           </cell>
           <cell r="I19">
             <v>0</v>
@@ -12236,7 +12238,7 @@
             <v>538</v>
           </cell>
           <cell r="H20">
-            <v>255</v>
+            <v>508</v>
           </cell>
           <cell r="I20">
             <v>0</v>
@@ -12274,7 +12276,7 @@
             <v>525763.644</v>
           </cell>
           <cell r="H21">
-            <v>239297.004</v>
+            <v>1477637.646</v>
           </cell>
           <cell r="I21">
             <v>0</v>
@@ -12299,7 +12301,9 @@
       <sheetData sheetId="3"/>
       <sheetData sheetId="4"/>
       <sheetData sheetId="5"/>
-      <sheetData sheetId="6">
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8">
         <row r="4">
           <cell r="B4">
             <v>329446.831260062</v>
@@ -12453,7 +12457,7 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="7">
+      <sheetData sheetId="9">
         <row r="4">
           <cell r="B4">
             <v>116176.256</v>
@@ -12607,10 +12611,10 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
       <sheetData sheetId="10"/>
       <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -23232,7 +23236,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{def1cc48-045d-43d8-911d-da0189b8d53a}</x14:id>
+          <x14:id>{117c2b93-a60a-4a25-9dd0-93c5e1f7dbf1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23246,7 +23250,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{27dc84f6-5264-4585-9322-c916ee6a8210}</x14:id>
+          <x14:id>{ea7742eb-0e4d-4887-baae-9e01446756cd}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23260,7 +23264,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{e4cd20b2-5914-45be-89d0-9ebe5a7bccfb}</x14:id>
+          <x14:id>{e697a7aa-e418-4ca3-8e70-0f35776a97ee}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23274,7 +23278,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1d7a31d5-2187-4d56-9aae-4b4cd1960308}</x14:id>
+          <x14:id>{2a4e78df-eb44-4c8c-858a-3cefda83aa18}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23288,7 +23292,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9b0a9a7a-a9d7-41e5-83ae-135f858be01c}</x14:id>
+          <x14:id>{6d284893-33f1-4e8b-b784-60f3f93efa07}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23302,7 +23306,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{af12d1fb-72e9-42b8-a6dc-aa2115b1596c}</x14:id>
+          <x14:id>{6281bfaa-98df-49e9-8a3d-422c35beec31}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23316,7 +23320,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5f2166c8-1a61-4cde-96cf-122c6218227b}</x14:id>
+          <x14:id>{d213ffdc-b40b-46aa-a5e7-17467f5580da}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23330,7 +23334,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2330c03d-92eb-4eb6-aaaa-ed153cf3527f}</x14:id>
+          <x14:id>{659fbe50-33e6-4308-baeb-d0bfe5ea5d91}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23350,7 +23354,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2b089e82-d75a-4b9b-863e-d67d565143c0}</x14:id>
+          <x14:id>{ec9ec053-6965-45db-869b-dc7b0782c0e7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23378,7 +23382,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7863629a-2b10-4a75-b9b9-5b00bb73b2bb}</x14:id>
+          <x14:id>{ab0370ef-9ca9-42cf-bf3c-32f563c7b620}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23398,7 +23402,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{77b48896-8834-49ae-ac67-a03268417c86}</x14:id>
+          <x14:id>{a00ccc80-937f-4fc0-9044-fa43ac37d21d}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23426,7 +23430,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{82a1a8e8-a8a2-4e8d-a3eb-4a37deaa259c}</x14:id>
+          <x14:id>{066f3225-4539-4d51-a535-1ff4e0015520}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23446,7 +23450,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3ea12327-1484-4ca7-a2a3-3b9830597acd}</x14:id>
+          <x14:id>{6f7a4333-d9a1-48e8-84a2-92a61a2f200e}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23474,7 +23478,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d365cafd-d987-4ecc-945c-e7ffbbd5a8b0}</x14:id>
+          <x14:id>{e5b36c51-12a6-4310-9b86-229631f65e79}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23494,7 +23498,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8bd1842e-6765-42ae-a3e0-7940c878a0ef}</x14:id>
+          <x14:id>{4062795d-10b5-4010-967f-24eb362789a4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23522,7 +23526,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{fa50584f-8e2a-4b7d-ae43-4d4868eff7d6}</x14:id>
+          <x14:id>{5706d3c5-75c6-4fa7-a655-adad25dfa543}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23542,7 +23546,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{b92da82f-36b3-44d4-aee1-78931aebe406}</x14:id>
+          <x14:id>{7b98a000-f68f-4323-bc3e-5415402d21c2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23570,7 +23574,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{10f03b71-5b7d-4bb1-8af3-e0d920219dd4}</x14:id>
+          <x14:id>{aa292887-1b6c-4e8f-bc6d-e4edba523bf2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23632,7 +23636,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6e8f3f5a-0882-4fb4-8c12-2056c4a2c449}</x14:id>
+          <x14:id>{03050f35-5fa8-49ab-90db-6ea4cd66d143}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23662,7 +23666,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{fabd9b76-78bf-4952-852e-e1addfeee7ea}</x14:id>
+          <x14:id>{d6e3c6bc-1679-4438-9772-b8341ac2c202}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23684,7 +23688,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{a7d26abd-6200-4fdb-84ba-174470d2f519}</x14:id>
+          <x14:id>{90942f48-2728-41b5-920d-0e7519cdadb4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23704,7 +23708,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{374dc5d8-438a-442e-80e4-25b2421ed0ea}</x14:id>
+          <x14:id>{181df0e5-e86f-4a43-b4e9-7c4af8501bf1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23726,7 +23730,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{f53c3f17-0e88-4052-aefc-4859cbd0f674}</x14:id>
+          <x14:id>{de28e55f-2cb9-4aec-b80a-ba262948dc68}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23746,7 +23750,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{e843d7c6-c2fa-4440-b740-2b7932f00a00}</x14:id>
+          <x14:id>{3d444d55-2306-4b0c-a863-2ca378005cc2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23768,7 +23772,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{c21e2b1c-b01c-41c4-b1da-65f2f286ce6c}</x14:id>
+          <x14:id>{88c7cc0d-62b0-4ff5-820f-80584bf2f131}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23788,7 +23792,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{941253e4-f0ed-4b6d-983f-5cace3e58429}</x14:id>
+          <x14:id>{30c06539-f1e8-4fa7-9a41-e7c7967ef56b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23810,7 +23814,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5efcbe13-516c-4e0d-9a50-85f0134b8107}</x14:id>
+          <x14:id>{d5c87590-9373-43b1-89f0-ad6700ea1ab4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23830,7 +23834,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{93bc68f4-b29e-44f8-8618-f5ee45dd230f}</x14:id>
+          <x14:id>{0c416cb5-a6be-479d-a740-1e1b457b97ca}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23858,7 +23862,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2647211d-7189-4de4-b029-cfefd999b4bd}</x14:id>
+          <x14:id>{bcf0736e-e2bc-495a-840c-da24b0e48a26}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23872,7 +23876,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{a2ab54dd-a64a-496e-920d-8a26239ffa7a}</x14:id>
+          <x14:id>{af6db539-97de-4b7d-a27d-b21627edd6da}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23902,7 +23906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d90a73b3-2459-47b8-b09b-981ae88f4091}</x14:id>
+          <x14:id>{c73c7343-4005-4e88-a0c8-3d88168d3033}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23924,7 +23928,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{917aa60c-8061-4e98-925e-b24e0ec135f1}</x14:id>
+          <x14:id>{6f69c397-d159-4601-b543-d21940b90cdd}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23946,7 +23950,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{917002c4-af57-4690-9927-c5a2432352c7}</x14:id>
+          <x14:id>{92380221-cf61-4e12-ac75-43ac6789d333}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23968,7 +23972,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8fcc5889-6eaa-4c4d-87da-55b54ab2df25}</x14:id>
+          <x14:id>{f516020c-25ba-48e6-a18b-57813749c74d}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23990,7 +23994,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{71ad9c27-4f7d-4192-af46-ef2b78004183}</x14:id>
+          <x14:id>{a463bfae-5e5f-42aa-af8a-89ea0ea8ee1f}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24012,7 +24016,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9d3c53b1-0334-4a84-9b83-1f6960e679f0}</x14:id>
+          <x14:id>{ef902de2-1c17-4ee2-bde3-e6d888c17457}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24034,7 +24038,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3c4c1ab1-5ba6-4c32-a846-d16fc750c010}</x14:id>
+          <x14:id>{6f8f211b-9ceb-4c17-9d59-a2f67856f62b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24056,7 +24060,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{108b2412-fd92-4673-9a32-aa76fb093f32}</x14:id>
+          <x14:id>{f264de6a-ebfc-4b25-b796-39300e5c3144}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24078,7 +24082,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ec1fa653-4925-4a1a-b9e8-6e2db966f925}</x14:id>
+          <x14:id>{6a4e437a-e3a5-4069-832b-130d6ce1f19b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24100,7 +24104,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4638a353-201f-4f30-b760-3bab4f315afb}</x14:id>
+          <x14:id>{3cdfad12-35de-45d0-9e82-91a943903eb0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24122,7 +24126,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{badfdc39-a2cd-4972-9578-9f83d5ec36f4}</x14:id>
+          <x14:id>{fe0ea55e-e848-447e-af72-e7c9256ac807}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24144,7 +24148,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{c874ea18-6939-4fe6-af69-f2fac0f44c53}</x14:id>
+          <x14:id>{8a088045-f7d2-427b-8ae5-b8c6a0ebd2ee}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24166,7 +24170,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{42b014e9-01ce-4835-9fdc-cba3990bcdf0}</x14:id>
+          <x14:id>{0e872a57-b5cb-4173-9d46-b0dad59e0d47}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24185,7 +24189,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{def1cc48-045d-43d8-911d-da0189b8d53a}">
+          <x14:cfRule type="dataBar" id="{117c2b93-a60a-4a25-9dd0-93c5e1f7dbf1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24198,7 +24202,7 @@
           <xm:sqref>C8:O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{27dc84f6-5264-4585-9322-c916ee6a8210}">
+          <x14:cfRule type="dataBar" id="{ea7742eb-0e4d-4887-baae-9e01446756cd}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24211,7 +24215,7 @@
           <xm:sqref>C12:O12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{e4cd20b2-5914-45be-89d0-9ebe5a7bccfb}">
+          <x14:cfRule type="dataBar" id="{e697a7aa-e418-4ca3-8e70-0f35776a97ee}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24224,7 +24228,7 @@
           <xm:sqref>C16:O16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1d7a31d5-2187-4d56-9aae-4b4cd1960308}">
+          <x14:cfRule type="dataBar" id="{2a4e78df-eb44-4c8c-858a-3cefda83aa18}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24237,7 +24241,7 @@
           <xm:sqref>C20:O20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9b0a9a7a-a9d7-41e5-83ae-135f858be01c}">
+          <x14:cfRule type="dataBar" id="{6d284893-33f1-4e8b-b784-60f3f93efa07}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24250,7 +24254,7 @@
           <xm:sqref>C24:O24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{af12d1fb-72e9-42b8-a6dc-aa2115b1596c}">
+          <x14:cfRule type="dataBar" id="{6281bfaa-98df-49e9-8a3d-422c35beec31}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24263,7 +24267,7 @@
           <xm:sqref>C27:O27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5f2166c8-1a61-4cde-96cf-122c6218227b}">
+          <x14:cfRule type="dataBar" id="{d213ffdc-b40b-46aa-a5e7-17467f5580da}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24276,7 +24280,7 @@
           <xm:sqref>C36:O36</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2330c03d-92eb-4eb6-aaaa-ed153cf3527f}">
+          <x14:cfRule type="dataBar" id="{659fbe50-33e6-4308-baeb-d0bfe5ea5d91}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24289,7 +24293,7 @@
           <xm:sqref>C44:N44</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2b089e82-d75a-4b9b-863e-d67d565143c0}">
+          <x14:cfRule type="dataBar" id="{ec9ec053-6965-45db-869b-dc7b0782c0e7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24302,7 +24306,7 @@
           <xm:sqref>O44</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7863629a-2b10-4a75-b9b9-5b00bb73b2bb}">
+          <x14:cfRule type="dataBar" id="{ab0370ef-9ca9-42cf-bf3c-32f563c7b620}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24315,7 +24319,7 @@
           <xm:sqref>C52:N52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{77b48896-8834-49ae-ac67-a03268417c86}">
+          <x14:cfRule type="dataBar" id="{a00ccc80-937f-4fc0-9044-fa43ac37d21d}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24328,7 +24332,7 @@
           <xm:sqref>O52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{82a1a8e8-a8a2-4e8d-a3eb-4a37deaa259c}">
+          <x14:cfRule type="dataBar" id="{066f3225-4539-4d51-a535-1ff4e0015520}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24341,7 +24345,7 @@
           <xm:sqref>C60:N60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3ea12327-1484-4ca7-a2a3-3b9830597acd}">
+          <x14:cfRule type="dataBar" id="{6f7a4333-d9a1-48e8-84a2-92a61a2f200e}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24354,7 +24358,7 @@
           <xm:sqref>O60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d365cafd-d987-4ecc-945c-e7ffbbd5a8b0}">
+          <x14:cfRule type="dataBar" id="{e5b36c51-12a6-4310-9b86-229631f65e79}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24367,7 +24371,7 @@
           <xm:sqref>C68:N68</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8bd1842e-6765-42ae-a3e0-7940c878a0ef}">
+          <x14:cfRule type="dataBar" id="{4062795d-10b5-4010-967f-24eb362789a4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24380,7 +24384,7 @@
           <xm:sqref>O68</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{fa50584f-8e2a-4b7d-ae43-4d4868eff7d6}">
+          <x14:cfRule type="dataBar" id="{5706d3c5-75c6-4fa7-a655-adad25dfa543}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24393,7 +24397,7 @@
           <xm:sqref>C76:N76</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{b92da82f-36b3-44d4-aee1-78931aebe406}">
+          <x14:cfRule type="dataBar" id="{7b98a000-f68f-4323-bc3e-5415402d21c2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24406,7 +24410,7 @@
           <xm:sqref>O76</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{10f03b71-5b7d-4bb1-8af3-e0d920219dd4}">
+          <x14:cfRule type="dataBar" id="{aa292887-1b6c-4e8f-bc6d-e4edba523bf2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24419,7 +24423,7 @@
           <xm:sqref>C132:O132</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6e8f3f5a-0882-4fb4-8c12-2056c4a2c449}">
+          <x14:cfRule type="dataBar" id="{03050f35-5fa8-49ab-90db-6ea4cd66d143}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24432,7 +24436,7 @@
           <xm:sqref>C26:O26 D27:N27 C28:O28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{fabd9b76-78bf-4952-852e-e1addfeee7ea}">
+          <x14:cfRule type="dataBar" id="{d6e3c6bc-1679-4438-9772-b8341ac2c202}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24445,7 +24449,7 @@
           <xm:sqref>C35:O35 D36:N36 C37:O37</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{a7d26abd-6200-4fdb-84ba-174470d2f519}">
+          <x14:cfRule type="dataBar" id="{90942f48-2728-41b5-920d-0e7519cdadb4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24458,7 +24462,7 @@
           <xm:sqref>C43:N43 D44:N44 C45:N45</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{374dc5d8-438a-442e-80e4-25b2421ed0ea}">
+          <x14:cfRule type="dataBar" id="{181df0e5-e86f-4a43-b4e9-7c4af8501bf1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24471,7 +24475,7 @@
           <xm:sqref>O43 O45</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{f53c3f17-0e88-4052-aefc-4859cbd0f674}">
+          <x14:cfRule type="dataBar" id="{de28e55f-2cb9-4aec-b80a-ba262948dc68}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24484,7 +24488,7 @@
           <xm:sqref>C51:N51 D52:N52 C53:N53</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{e843d7c6-c2fa-4440-b740-2b7932f00a00}">
+          <x14:cfRule type="dataBar" id="{3d444d55-2306-4b0c-a863-2ca378005cc2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24497,7 +24501,7 @@
           <xm:sqref>O51 O53</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{c21e2b1c-b01c-41c4-b1da-65f2f286ce6c}">
+          <x14:cfRule type="dataBar" id="{88c7cc0d-62b0-4ff5-820f-80584bf2f131}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24510,7 +24514,7 @@
           <xm:sqref>C59:N59 D60:N60 C61:N61</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{941253e4-f0ed-4b6d-983f-5cace3e58429}">
+          <x14:cfRule type="dataBar" id="{30c06539-f1e8-4fa7-9a41-e7c7967ef56b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24523,7 +24527,7 @@
           <xm:sqref>O59 O61</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5efcbe13-516c-4e0d-9a50-85f0134b8107}">
+          <x14:cfRule type="dataBar" id="{d5c87590-9373-43b1-89f0-ad6700ea1ab4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24536,7 +24540,7 @@
           <xm:sqref>C67:N67 D68:N68 C69:N69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{93bc68f4-b29e-44f8-8618-f5ee45dd230f}">
+          <x14:cfRule type="dataBar" id="{0c416cb5-a6be-479d-a740-1e1b457b97ca}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24549,7 +24553,7 @@
           <xm:sqref>O67 O69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2647211d-7189-4de4-b029-cfefd999b4bd}">
+          <x14:cfRule type="dataBar" id="{bcf0736e-e2bc-495a-840c-da24b0e48a26}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24562,7 +24566,7 @@
           <xm:sqref>C75:N75 D76:N76 C77:N77</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{a2ab54dd-a64a-496e-920d-8a26239ffa7a}">
+          <x14:cfRule type="dataBar" id="{af6db539-97de-4b7d-a27d-b21627edd6da}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24575,7 +24579,7 @@
           <xm:sqref>O75 O77</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d90a73b3-2459-47b8-b09b-981ae88f4091}">
+          <x14:cfRule type="dataBar" id="{c73c7343-4005-4e88-a0c8-3d88168d3033}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24588,7 +24592,7 @@
           <xm:sqref>C83:N83 D84:N84 C85:O85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{917aa60c-8061-4e98-925e-b24e0ec135f1}">
+          <x14:cfRule type="dataBar" id="{6f69c397-d159-4601-b543-d21940b90cdd}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24601,7 +24605,7 @@
           <xm:sqref>C84:O84 D85:N85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{917002c4-af57-4690-9927-c5a2432352c7}">
+          <x14:cfRule type="dataBar" id="{92380221-cf61-4e12-ac75-43ac6789d333}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24614,7 +24618,7 @@
           <xm:sqref>C91:N91 D92:N92 C93:O93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8fcc5889-6eaa-4c4d-87da-55b54ab2df25}">
+          <x14:cfRule type="dataBar" id="{f516020c-25ba-48e6-a18b-57813749c74d}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24627,7 +24631,7 @@
           <xm:sqref>C92:O92 D93:N93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{71ad9c27-4f7d-4192-af46-ef2b78004183}">
+          <x14:cfRule type="dataBar" id="{a463bfae-5e5f-42aa-af8a-89ea0ea8ee1f}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24640,7 +24644,7 @@
           <xm:sqref>C99:N99 D100:N100 C101:O101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9d3c53b1-0334-4a84-9b83-1f6960e679f0}">
+          <x14:cfRule type="dataBar" id="{ef902de2-1c17-4ee2-bde3-e6d888c17457}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24653,7 +24657,7 @@
           <xm:sqref>C100:O100 D101:N101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3c4c1ab1-5ba6-4c32-a846-d16fc750c010}">
+          <x14:cfRule type="dataBar" id="{6f8f211b-9ceb-4c17-9d59-a2f67856f62b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24666,7 +24670,7 @@
           <xm:sqref>C107:N107 D108:N108 C109:O109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{108b2412-fd92-4673-9a32-aa76fb093f32}">
+          <x14:cfRule type="dataBar" id="{f264de6a-ebfc-4b25-b796-39300e5c3144}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24679,7 +24683,7 @@
           <xm:sqref>C108:O108 D109:N109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ec1fa653-4925-4a1a-b9e8-6e2db966f925}">
+          <x14:cfRule type="dataBar" id="{6a4e437a-e3a5-4069-832b-130d6ce1f19b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24692,7 +24696,7 @@
           <xm:sqref>C115:N115 D116:N116 C117:O117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4638a353-201f-4f30-b760-3bab4f315afb}">
+          <x14:cfRule type="dataBar" id="{3cdfad12-35de-45d0-9e82-91a943903eb0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24705,7 +24709,7 @@
           <xm:sqref>C116:O116 D117:N117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{badfdc39-a2cd-4972-9578-9f83d5ec36f4}">
+          <x14:cfRule type="dataBar" id="{fe0ea55e-e848-447e-af72-e7c9256ac807}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24718,7 +24722,7 @@
           <xm:sqref>C123:N123 D124:N124 C125:O125</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{c874ea18-6939-4fe6-af69-f2fac0f44c53}">
+          <x14:cfRule type="dataBar" id="{8a088045-f7d2-427b-8ae5-b8c6a0ebd2ee}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24731,7 +24735,7 @@
           <xm:sqref>C124:O124 D125:N125</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{42b014e9-01ce-4835-9fdc-cba3990bcdf0}">
+          <x14:cfRule type="dataBar" id="{0e872a57-b5cb-4173-9d46-b0dad59e0d47}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24965,7 +24969,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="3">
         <f>(F7+G7+H7)</f>
-        <v>621223.21</v>
+        <v>748705.97</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -25003,7 +25007,7 @@
       <c r="E5" s="5"/>
       <c r="F5" s="6">
         <f>(F7+G7+H7)/(F6+G6+H6)</f>
-        <v>1.08038464388486</v>
+        <v>1.30209306373617</v>
       </c>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -25118,7 +25122,7 @@
       </c>
       <c r="H7" s="12">
         <f>'[2]2026年月度数据汇总--俄罗斯'!H13+'[2]2026年月度数据汇总--俄罗斯'!H18</f>
-        <v>144320.02</v>
+        <v>271802.78</v>
       </c>
       <c r="I7" s="12">
         <f>'[2]2026年月度数据汇总--俄罗斯'!I13+'[2]2026年月度数据汇总--俄罗斯'!I18</f>
@@ -25146,7 +25150,7 @@
       </c>
       <c r="O7" s="12">
         <f t="shared" si="0"/>
-        <v>911007.01</v>
+        <v>1038489.77</v>
       </c>
     </row>
     <row r="8" ht="15.6" spans="1:15">
@@ -25180,7 +25184,7 @@
       </c>
       <c r="H8" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H8</f>
-        <v>0.535748473942456</v>
+        <v>1.05062851406593</v>
       </c>
       <c r="I8" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I8</f>
@@ -25208,7 +25212,7 @@
       </c>
       <c r="O8" s="20">
         <f>O7/O6</f>
-        <v>0.297266079069626</v>
+        <v>0.338864332209494</v>
       </c>
     </row>
     <row r="9" ht="15.6" spans="1:15">
@@ -25366,7 +25370,7 @@
       </c>
       <c r="H11" s="11">
         <f>'[2]2026年月度数据汇总--俄罗斯'!H14+'[2]2026年月度数据汇总--俄罗斯'!H19</f>
-        <v>6094</v>
+        <v>12016</v>
       </c>
       <c r="I11" s="11">
         <f>'[2]2026年月度数据汇总--俄罗斯'!I14+'[2]2026年月度数据汇总--俄罗斯'!I19</f>
@@ -25394,7 +25398,7 @@
       </c>
       <c r="O11" s="11">
         <f t="shared" si="0"/>
-        <v>51471</v>
+        <v>57393</v>
       </c>
     </row>
     <row r="12" ht="15.6" spans="1:15">
@@ -25428,7 +25432,7 @@
       </c>
       <c r="H12" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H12</f>
-        <v>0.395130201208745</v>
+        <v>0.814808366702315</v>
       </c>
       <c r="I12" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I12</f>
@@ -25456,7 +25460,7 @@
       </c>
       <c r="O12" s="20">
         <f>O11/O10</f>
-        <v>0.249580565388159</v>
+        <v>0.278296077195364</v>
       </c>
     </row>
     <row r="13" ht="15.6" spans="1:15">
@@ -25614,7 +25618,7 @@
       </c>
       <c r="H15" s="11">
         <f>'[2]2026年月度数据汇总--俄罗斯'!H15+'[2]2026年月度数据汇总--俄罗斯'!H20</f>
-        <v>2249</v>
+        <v>4596</v>
       </c>
       <c r="I15" s="11">
         <f>'[2]2026年月度数据汇总--俄罗斯'!I15+'[2]2026年月度数据汇总--俄罗斯'!I20</f>
@@ -25642,7 +25646,7 @@
       </c>
       <c r="O15" s="11">
         <f t="shared" si="1"/>
-        <v>18251</v>
+        <v>20598</v>
       </c>
     </row>
     <row r="16" ht="15.6" spans="1:15">
@@ -25676,7 +25680,7 @@
       </c>
       <c r="H16" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H16</f>
-        <v>0.441264841541795</v>
+        <v>0.919275009888344</v>
       </c>
       <c r="I16" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I16</f>
@@ -25704,7 +25708,7 @@
       </c>
       <c r="O16" s="20">
         <f>O15/O14</f>
-        <v>0.28547831813212</v>
+        <v>0.322189600399178</v>
       </c>
     </row>
     <row r="17" ht="15.6" spans="1:15">
@@ -25862,7 +25866,7 @@
       </c>
       <c r="H19" s="19">
         <f>'[2]2026年月度数据汇总--俄罗斯'!H16+'[2]2026年月度数据汇总--俄罗斯'!H21</f>
-        <v>2513446.9992</v>
+        <v>6073636.7304</v>
       </c>
       <c r="I19" s="19">
         <f>'[2]2026年月度数据汇总--俄罗斯'!I16+'[2]2026年月度数据汇总--俄罗斯'!I21</f>
@@ -25890,7 +25894,7 @@
       </c>
       <c r="O19" s="19">
         <f t="shared" si="1"/>
-        <v>19421438.5959</v>
+        <v>22981628.3271</v>
       </c>
     </row>
     <row r="20" ht="15.6" spans="1:15">
@@ -25924,7 +25928,7 @@
       </c>
       <c r="H20" s="20">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H20</f>
-        <v>0.476369032961964</v>
+        <v>1.07917936735439</v>
       </c>
       <c r="I20" s="20">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I20</f>
@@ -25952,7 +25956,7 @@
       </c>
       <c r="O20" s="20">
         <f>O19/O18</f>
-        <v>0.0218389196449133</v>
+        <v>0.0258422635309186</v>
       </c>
     </row>
     <row r="21" ht="15.6" spans="1:15">
@@ -26026,21 +26030,57 @@
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!B22</f>
         <v>GSV目标</v>
       </c>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="21"/>
-      <c r="L22" s="21"/>
-      <c r="M22" s="21"/>
-      <c r="N22" s="21"/>
+      <c r="C22" s="21">
+        <f t="shared" ref="C22:N22" si="2">C18*(1-0.68)/12.5</f>
+        <v>837939.2</v>
+      </c>
+      <c r="D22" s="21">
+        <f t="shared" si="2"/>
+        <v>876928</v>
+      </c>
+      <c r="E22" s="21">
+        <f t="shared" si="2"/>
+        <v>787968</v>
+      </c>
+      <c r="F22" s="21">
+        <f t="shared" si="2"/>
+        <v>1140403.2</v>
+      </c>
+      <c r="G22" s="21">
+        <f t="shared" si="2"/>
+        <v>1497600</v>
+      </c>
+      <c r="H22" s="21">
+        <f t="shared" si="2"/>
+        <v>1722112</v>
+      </c>
+      <c r="I22" s="21">
+        <f t="shared" si="2"/>
+        <v>2071296</v>
+      </c>
+      <c r="J22" s="21">
+        <f t="shared" si="2"/>
+        <v>2657280</v>
+      </c>
+      <c r="K22" s="21">
+        <f t="shared" si="2"/>
+        <v>3420416</v>
+      </c>
+      <c r="L22" s="21">
+        <f t="shared" si="2"/>
+        <v>3310080</v>
+      </c>
+      <c r="M22" s="21">
+        <f t="shared" si="2"/>
+        <v>2722048</v>
+      </c>
+      <c r="N22" s="21">
+        <f t="shared" si="2"/>
+        <v>1722112</v>
+      </c>
       <c r="O22" s="28">
         <f>SUM(C22:N22)</f>
-        <v>0</v>
+        <v>22766182.4</v>
       </c>
     </row>
     <row r="23" ht="15.6" spans="1:15">
@@ -26090,9 +26130,9 @@
       <c r="L24" s="13"/>
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
-      <c r="O24" s="20" t="e">
+      <c r="O24" s="20">
         <f>O23/O22</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" ht="15.6" spans="1:15">
@@ -26167,55 +26207,55 @@
         <v>退款率</v>
       </c>
       <c r="C26" s="13">
-        <f t="shared" ref="C26:O26" si="2">1-C23/C19</f>
+        <f t="shared" ref="C26:O26" si="3">1-C23/C19</f>
         <v>1</v>
       </c>
       <c r="D26" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="E26" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="F26" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="G26" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="H26" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="I26" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="J26" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="K26" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="L26" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="M26" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="N26" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O26" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
     </row>
@@ -26229,56 +26269,56 @@
         <v>退货率</v>
       </c>
       <c r="C27" s="13">
-        <f t="shared" ref="C27:O27" si="3">1-C15/C11</f>
+        <f t="shared" ref="C27:O27" si="4">1-C15/C11</f>
         <v>0.669214234535467</v>
       </c>
       <c r="D27" s="13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.652624388022316</v>
       </c>
       <c r="E27" s="13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.641507259737267</v>
       </c>
       <c r="F27" s="13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.657728543327467</v>
       </c>
       <c r="G27" s="13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.619143984620055</v>
       </c>
       <c r="H27" s="13">
-        <f t="shared" si="3"/>
-        <v>0.630948473908763</v>
+        <f t="shared" si="4"/>
+        <v>0.617509986684421</v>
       </c>
       <c r="I27" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="J27" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="K27" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="L27" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="M27" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="N27" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O27" s="13">
-        <f t="shared" si="3"/>
-        <v>0.645411979561306</v>
+        <f t="shared" si="4"/>
+        <v>0.641106058230098</v>
       </c>
     </row>
     <row r="28" ht="15.6" spans="1:15">
@@ -26291,55 +26331,55 @@
         <v>利润率</v>
       </c>
       <c r="C28" s="13" t="e">
-        <f t="shared" ref="C28:O28" si="4">C7/(C23)</f>
+        <f t="shared" ref="C28:O28" si="5">C7/(C23)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="D28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="E28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="F28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="G28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="H28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="J28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="K28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="L28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="M28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="N28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O28" s="13" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -26457,7 +26497,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{aa3f6560-21eb-4bec-b6bf-5697438d3315}</x14:id>
+          <x14:id>{6634a2ee-9569-4702-b8de-2e31e21badd1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26471,7 +26511,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5508a77f-be2a-48f2-b9be-0e6bbed65b3f}</x14:id>
+          <x14:id>{9fbe3b44-541c-4d35-a062-3ebf92894c91}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26485,7 +26525,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{abc651fb-f841-4002-8141-d0aafe044223}</x14:id>
+          <x14:id>{8fc3673c-c48e-466f-92ff-fe7e91c36a09}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26499,7 +26539,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d45611b3-9398-47a5-8d66-7d7ffd04e28a}</x14:id>
+          <x14:id>{e5f3b597-ad35-4c00-b38e-d584b7d9f0c6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26513,7 +26553,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{479cb120-c7a1-47d9-8054-9319d9afc2d1}</x14:id>
+          <x14:id>{0fe407a0-2d01-4d45-b703-e4359ffd8b19}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26527,7 +26567,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{120941f6-55a5-4ce2-bdc0-7315c227d67c}</x14:id>
+          <x14:id>{8df41d9e-53c5-4eed-850c-241e99e92f48}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26541,7 +26581,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{faa45d6d-6d93-4910-b3d6-2e11083f0ce2}</x14:id>
+          <x14:id>{636b744f-e9d8-4e94-8971-7b327f5fa816}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26555,7 +26595,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3a45acb7-e203-468f-8977-00729cbd63af}</x14:id>
+          <x14:id>{b823a50f-9d1a-43de-ae60-3c64a2e52a4e}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26569,7 +26609,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{66c5a367-f219-4d73-8cf3-4d54c632e705}</x14:id>
+          <x14:id>{067185f9-d18b-4454-b881-32d76c5ae9b8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26583,7 +26623,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d4836457-0298-49b1-90a3-d9f221954a6d}</x14:id>
+          <x14:id>{37d1ce29-b0b5-4b7d-a78d-ab7d2228db9b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26597,7 +26637,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{c016f0db-e482-4ee1-aa34-c736ea3f0249}</x14:id>
+          <x14:id>{f9b9c13c-6ea6-41b7-9628-026f56abc497}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26633,7 +26673,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4fdd3c22-1eb5-4837-9182-96ad2305f63d}</x14:id>
+          <x14:id>{20866eed-a0ea-488f-aa87-700358517c8a}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26652,7 +26692,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{aa3f6560-21eb-4bec-b6bf-5697438d3315}">
+          <x14:cfRule type="dataBar" id="{6634a2ee-9569-4702-b8de-2e31e21badd1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26665,7 +26705,7 @@
           <xm:sqref>C8:N8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5508a77f-be2a-48f2-b9be-0e6bbed65b3f}">
+          <x14:cfRule type="dataBar" id="{9fbe3b44-541c-4d35-a062-3ebf92894c91}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26678,7 +26718,7 @@
           <xm:sqref>O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{abc651fb-f841-4002-8141-d0aafe044223}">
+          <x14:cfRule type="dataBar" id="{8fc3673c-c48e-466f-92ff-fe7e91c36a09}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26691,7 +26731,7 @@
           <xm:sqref>C12:N12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d45611b3-9398-47a5-8d66-7d7ffd04e28a}">
+          <x14:cfRule type="dataBar" id="{e5f3b597-ad35-4c00-b38e-d584b7d9f0c6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26704,7 +26744,7 @@
           <xm:sqref>O12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{479cb120-c7a1-47d9-8054-9319d9afc2d1}">
+          <x14:cfRule type="dataBar" id="{0fe407a0-2d01-4d45-b703-e4359ffd8b19}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26717,7 +26757,7 @@
           <xm:sqref>C16:N16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{120941f6-55a5-4ce2-bdc0-7315c227d67c}">
+          <x14:cfRule type="dataBar" id="{8df41d9e-53c5-4eed-850c-241e99e92f48}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26730,7 +26770,7 @@
           <xm:sqref>O16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{faa45d6d-6d93-4910-b3d6-2e11083f0ce2}">
+          <x14:cfRule type="dataBar" id="{636b744f-e9d8-4e94-8971-7b327f5fa816}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26743,7 +26783,7 @@
           <xm:sqref>B20:N20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3a45acb7-e203-468f-8977-00729cbd63af}">
+          <x14:cfRule type="dataBar" id="{b823a50f-9d1a-43de-ae60-3c64a2e52a4e}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26756,7 +26796,7 @@
           <xm:sqref>O20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{66c5a367-f219-4d73-8cf3-4d54c632e705}">
+          <x14:cfRule type="dataBar" id="{067185f9-d18b-4454-b881-32d76c5ae9b8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26769,7 +26809,7 @@
           <xm:sqref>C24:N24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d4836457-0298-49b1-90a3-d9f221954a6d}">
+          <x14:cfRule type="dataBar" id="{37d1ce29-b0b5-4b7d-a78d-ab7d2228db9b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26782,7 +26822,7 @@
           <xm:sqref>O24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{c016f0db-e482-4ee1-aa34-c736ea3f0249}">
+          <x14:cfRule type="dataBar" id="{f9b9c13c-6ea6-41b7-9628-026f56abc497}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26795,7 +26835,7 @@
           <xm:sqref>C27:O27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4fdd3c22-1eb5-4837-9182-96ad2305f63d}">
+          <x14:cfRule type="dataBar" id="{20866eed-a0ea-488f-aa87-700358517c8a}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27030,7 +27070,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="3">
         <f>(F7+G7+H7)</f>
-        <v>1625199.49</v>
+        <v>1937577.24</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -27068,7 +27108,7 @@
       <c r="E5" s="5"/>
       <c r="F5" s="6">
         <f>(F7+G7+H7)/(F6+G6+H6)</f>
-        <v>1.00699686082307</v>
+        <v>1.20055058488987</v>
       </c>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -27183,7 +27223,7 @@
       </c>
       <c r="H7" s="12">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H7</f>
-        <v>325038.63</v>
+        <v>637416.38</v>
       </c>
       <c r="I7" s="12">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I7</f>
@@ -27211,7 +27251,7 @@
       </c>
       <c r="O7" s="12">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O7</f>
-        <v>3437257.96</v>
+        <v>3749635.71</v>
       </c>
     </row>
     <row r="8" s="37" customFormat="1" spans="1:15">
@@ -27245,7 +27285,7 @@
       </c>
       <c r="H8" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H8</f>
-        <v>0.535748473942456</v>
+        <v>1.05062851406593</v>
       </c>
       <c r="I8" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I8</f>
@@ -27273,7 +27313,7 @@
       </c>
       <c r="O8" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O8</f>
-        <v>0.392593009981998</v>
+        <v>0.428271833786046</v>
       </c>
     </row>
     <row r="9" s="37" customFormat="1" spans="1:15">
@@ -27431,7 +27471,7 @@
       </c>
       <c r="H11" s="11">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H11</f>
-        <v>15887</v>
+        <v>32761</v>
       </c>
       <c r="I11" s="11">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I11</f>
@@ -27459,7 +27499,7 @@
       </c>
       <c r="O11" s="11">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O11</f>
-        <v>171643</v>
+        <v>188517</v>
       </c>
     </row>
     <row r="12" s="37" customFormat="1" spans="1:15">
@@ -27493,7 +27533,7 @@
       </c>
       <c r="H12" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H12</f>
-        <v>0.395130201208745</v>
+        <v>0.814808366702315</v>
       </c>
       <c r="I12" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I12</f>
@@ -27521,7 +27561,7 @@
       </c>
       <c r="O12" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O12</f>
-        <v>0.295491950033742</v>
+        <v>0.324541379167872</v>
       </c>
     </row>
     <row r="13" s="37" customFormat="1" spans="1:15">
@@ -27679,7 +27719,7 @@
       </c>
       <c r="H15" s="11">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H15</f>
-        <v>5500</v>
+        <v>11458</v>
       </c>
       <c r="I15" s="11">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I15</f>
@@ -27707,7 +27747,7 @@
       </c>
       <c r="O15" s="11">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O15</f>
-        <v>60846</v>
+        <v>66804</v>
       </c>
     </row>
     <row r="16" s="37" customFormat="1" spans="1:15">
@@ -27741,7 +27781,7 @@
       </c>
       <c r="H16" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H16</f>
-        <v>0.441264841541795</v>
+        <v>0.919275009888344</v>
       </c>
       <c r="I16" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I16</f>
@@ -27769,7 +27809,7 @@
       </c>
       <c r="O16" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O16</f>
-        <v>0.337901326548428</v>
+        <v>0.370988400531526</v>
       </c>
     </row>
     <row r="17" s="37" customFormat="1" spans="1:15">
@@ -27927,7 +27967,7 @@
       </c>
       <c r="H19" s="22">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H19</f>
-        <v>6659288.4732</v>
+        <v>15086133.2796</v>
       </c>
       <c r="I19" s="22">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I19</f>
@@ -27955,7 +27995,7 @@
       </c>
       <c r="O19" s="12">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O19</f>
-        <v>67577309.1834</v>
+        <v>76004153.9898</v>
       </c>
     </row>
     <row r="20" s="37" customFormat="1" spans="1:15">
@@ -27989,7 +28029,7 @@
       </c>
       <c r="H20" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H20</f>
-        <v>0.476369032961964</v>
+        <v>1.07917936735439</v>
       </c>
       <c r="I20" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I20</f>
@@ -28017,7 +28057,7 @@
       </c>
       <c r="O20" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O20</f>
-        <v>0.335043434341862</v>
+        <v>0.376823124280976</v>
       </c>
     </row>
     <row r="21" s="37" customFormat="1" spans="1:15">
@@ -28175,7 +28215,7 @@
       </c>
       <c r="H23" s="22">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H23</f>
-        <v>1930982.2827</v>
+        <v>4076553.6474</v>
       </c>
       <c r="I23" s="22">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I23</f>
@@ -28203,7 +28243,7 @@
       </c>
       <c r="O23" s="12">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O23</f>
-        <v>21876883.9391</v>
+        <v>24022455.3038</v>
       </c>
     </row>
     <row r="24" s="37" customFormat="1" spans="1:15">
@@ -28237,7 +28277,7 @@
       </c>
       <c r="H24" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H24</f>
-        <v>0.431662184320827</v>
+        <v>0.911294768317202</v>
       </c>
       <c r="I24" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I24</f>
@@ -28265,7 +28305,7 @@
       </c>
       <c r="O24" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O24</f>
-        <v>0.33895004922076</v>
+        <v>0.372192512895943</v>
       </c>
     </row>
     <row r="25" s="37" customFormat="1" spans="1:15">
@@ -28361,7 +28401,7 @@
       </c>
       <c r="H26" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H26</f>
-        <v>0.289968258691773</v>
+        <v>0.270218588941704</v>
       </c>
       <c r="I26" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I26</f>
@@ -28389,7 +28429,7 @@
       </c>
       <c r="O26" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O26</f>
-        <v>0.323731208055765</v>
+        <v>0.316067662657279</v>
       </c>
     </row>
     <row r="27" s="37" customFormat="1" spans="1:15">
@@ -28423,7 +28463,7 @@
       </c>
       <c r="H27" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H27</f>
-        <v>0.653804997796941</v>
+        <v>0.65025487622478</v>
       </c>
       <c r="I27" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I27</f>
@@ -28451,7 +28491,7 @@
       </c>
       <c r="O27" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O27</f>
-        <v>0.645508409897287</v>
+        <v>0.645634080746033</v>
       </c>
     </row>
     <row r="28" s="37" customFormat="1" spans="1:15">
@@ -28485,7 +28525,7 @@
       </c>
       <c r="H28" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H28</f>
-        <v>0.168328126525073</v>
+        <v>0.156361582634032</v>
       </c>
       <c r="I28" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I28</f>
@@ -28513,7 +28553,7 @@
       </c>
       <c r="O28" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O28</f>
-        <v>0.157118260972107</v>
+        <v>0.156088778710595</v>
       </c>
     </row>
     <row r="29" s="37" customFormat="1" spans="1:15">
@@ -28609,7 +28649,7 @@
       </c>
       <c r="H30" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H30</f>
-        <v>102754.41</v>
+        <v>196174.75</v>
       </c>
       <c r="I30" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I30</f>
@@ -28637,7 +28677,7 @@
       </c>
       <c r="O30" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O30</f>
-        <v>1874915.07</v>
+        <v>1968335.41</v>
       </c>
     </row>
     <row r="31" s="37" customFormat="1" spans="1:15">
@@ -28671,7 +28711,7 @@
       </c>
       <c r="H31" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H31</f>
-        <v>5785</v>
+        <v>11621</v>
       </c>
       <c r="I31" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I31</f>
@@ -28699,7 +28739,7 @@
       </c>
       <c r="O31" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O31</f>
-        <v>82089</v>
+        <v>87925</v>
       </c>
     </row>
     <row r="32" s="37" customFormat="1" spans="1:15">
@@ -28733,7 +28773,7 @@
       </c>
       <c r="H32" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H32</f>
-        <v>1927</v>
+        <v>3917</v>
       </c>
       <c r="I32" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I32</f>
@@ -28761,7 +28801,7 @@
       </c>
       <c r="O32" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O32</f>
-        <v>30081</v>
+        <v>32071</v>
       </c>
     </row>
     <row r="33" s="37" customFormat="1" spans="1:15">
@@ -28795,7 +28835,7 @@
       </c>
       <c r="H33" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H33</f>
-        <v>2511111.222</v>
+        <v>5199070.2324</v>
       </c>
       <c r="I33" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I33</f>
@@ -28823,7 +28863,7 @@
       </c>
       <c r="O33" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O33</f>
-        <v>33826837.7889</v>
+        <v>36514796.7993</v>
       </c>
     </row>
     <row r="34" s="37" customFormat="1" spans="1:15">
@@ -28857,7 +28897,7 @@
       </c>
       <c r="H34" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H34</f>
-        <v>699411.4057</v>
+        <v>1456186.0782</v>
       </c>
       <c r="I34" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I34</f>
@@ -28885,7 +28925,7 @@
       </c>
       <c r="O34" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O34</f>
-        <v>11088070.4977</v>
+        <v>11844845.1702</v>
       </c>
     </row>
     <row r="35" s="37" customFormat="1" spans="1:15">
@@ -28919,7 +28959,7 @@
       </c>
       <c r="H35" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H35</f>
-        <v>0.278526653687186</v>
+        <v>0.280085864031076</v>
       </c>
       <c r="I35" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I35</f>
@@ -28947,7 +28987,7 @@
       </c>
       <c r="O35" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O35</f>
-        <v>0.327789152710528</v>
+        <v>0.324384803106095</v>
       </c>
     </row>
     <row r="36" s="37" customFormat="1" spans="1:15">
@@ -28981,7 +29021,7 @@
       </c>
       <c r="H36" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H36</f>
-        <v>0.666897147796024</v>
+        <v>0.662937785044316</v>
       </c>
       <c r="I36" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I36</f>
@@ -29009,7 +29049,7 @@
       </c>
       <c r="O36" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O36</f>
-        <v>0.633556262105763</v>
+        <v>0.635245948251351</v>
       </c>
     </row>
     <row r="37" s="37" customFormat="1" spans="1:15">
@@ -29043,7 +29083,7 @@
       </c>
       <c r="H37" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H37</f>
-        <v>0.1469155480774</v>
+        <v>0.134718188105804</v>
       </c>
       <c r="I37" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I37</f>
@@ -29071,7 +29111,7 @@
       </c>
       <c r="O37" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O37</f>
-        <v>0.169092996873434</v>
+        <v>0.166176541923238</v>
       </c>
     </row>
     <row r="38" s="37" customFormat="1" spans="1:15">
@@ -29105,7 +29145,7 @@
       </c>
       <c r="H38" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H38</f>
-        <v>77964.2</v>
+        <v>169438.85</v>
       </c>
       <c r="I38" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I38</f>
@@ -29133,7 +29173,7 @@
       </c>
       <c r="O38" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O38</f>
-        <v>651335.88</v>
+        <v>742810.53</v>
       </c>
     </row>
     <row r="39" s="37" customFormat="1" spans="1:15">
@@ -29167,7 +29207,7 @@
       </c>
       <c r="H39" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H39</f>
-        <v>4008</v>
+        <v>9124</v>
       </c>
       <c r="I39" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I39</f>
@@ -29195,7 +29235,7 @@
       </c>
       <c r="O39" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O39</f>
-        <v>38083</v>
+        <v>43199</v>
       </c>
     </row>
     <row r="40" s="37" customFormat="1" spans="1:15">
@@ -29229,7 +29269,7 @@
       </c>
       <c r="H40" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H40</f>
-        <v>1324</v>
+        <v>2945</v>
       </c>
       <c r="I40" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I40</f>
@@ -29257,7 +29297,7 @@
       </c>
       <c r="O40" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O40</f>
-        <v>12514</v>
+        <v>14135</v>
       </c>
     </row>
     <row r="41" s="37" customFormat="1" spans="1:15">
@@ -29291,7 +29331,7 @@
       </c>
       <c r="H41" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H41</f>
-        <v>1634730.252</v>
+        <v>3813426.3168</v>
       </c>
       <c r="I41" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I41</f>
@@ -29319,7 +29359,7 @@
       </c>
       <c r="O41" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O41</f>
-        <v>14329032.7986</v>
+        <v>16507728.8634</v>
       </c>
     </row>
     <row r="42" s="37" customFormat="1" spans="1:15">
@@ -29353,7 +29393,7 @@
       </c>
       <c r="H42" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H42</f>
-        <v>458423.5943</v>
+        <v>1032316.5394</v>
       </c>
       <c r="I42" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I42</f>
@@ -29381,7 +29421,7 @@
       </c>
       <c r="O42" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O42</f>
-        <v>4184008.9538</v>
+        <v>4757901.8989</v>
       </c>
     </row>
     <row r="43" s="37" customFormat="1" spans="1:15">
@@ -29415,7 +29455,7 @@
       </c>
       <c r="H43" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H43</f>
-        <v>0.280427669176089</v>
+        <v>0.270705778384164</v>
       </c>
       <c r="I43" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I43</f>
@@ -29443,7 +29483,7 @@
       </c>
       <c r="O43" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O43</f>
-        <v>0.291995210884631</v>
+        <v>0.288222682736748</v>
       </c>
     </row>
     <row r="44" s="37" customFormat="1" spans="1:15">
@@ -29477,7 +29517,7 @@
       </c>
       <c r="H44" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H44</f>
-        <v>0.669660678642715</v>
+        <v>0.677224901359053</v>
       </c>
       <c r="I44" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I44</f>
@@ -29505,7 +29545,7 @@
       </c>
       <c r="O44" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O44</f>
-        <v>0.671401937872542</v>
+        <v>0.672793351697956</v>
       </c>
     </row>
     <row r="45" s="37" customFormat="1" spans="1:15">
@@ -29539,7 +29579,7 @@
       </c>
       <c r="H45" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H45</f>
-        <v>0.170070216649841</v>
+        <v>0.164134588116239</v>
       </c>
       <c r="I45" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I45</f>
@@ -29567,7 +29607,7 @@
       </c>
       <c r="O45" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O45</f>
-        <v>0.155672678331255</v>
+        <v>0.156121447180686</v>
       </c>
     </row>
     <row r="46" s="37" customFormat="1" spans="1:15">
@@ -29601,7 +29641,7 @@
       </c>
       <c r="H46" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H46</f>
-        <v>131378.65</v>
+        <v>246129.6</v>
       </c>
       <c r="I46" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I46</f>
@@ -29629,7 +29669,7 @@
       </c>
       <c r="O46" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O46</f>
-        <v>764491.77</v>
+        <v>879242.72</v>
       </c>
     </row>
     <row r="47" s="37" customFormat="1" spans="1:15">
@@ -29663,7 +29703,7 @@
       </c>
       <c r="H47" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H47</f>
-        <v>5471</v>
+        <v>10835</v>
       </c>
       <c r="I47" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I47</f>
@@ -29691,7 +29731,7 @@
       </c>
       <c r="O47" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O47</f>
-        <v>34272</v>
+        <v>39636</v>
       </c>
     </row>
     <row r="48" s="37" customFormat="1" spans="1:15">
@@ -29725,7 +29765,7 @@
       </c>
       <c r="H48" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H48</f>
-        <v>1994</v>
+        <v>4088</v>
       </c>
       <c r="I48" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I48</f>
@@ -29753,7 +29793,7 @@
       </c>
       <c r="O48" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O48</f>
-        <v>11970</v>
+        <v>14064</v>
       </c>
     </row>
     <row r="49" s="37" customFormat="1" spans="1:15">
@@ -29787,7 +29827,7 @@
       </c>
       <c r="H49" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H49</f>
-        <v>2274149.9952</v>
+        <v>4595999.0844</v>
       </c>
       <c r="I49" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I49</f>
@@ -29815,7 +29855,7 @@
       </c>
       <c r="O49" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O49</f>
-        <v>13376634.4806</v>
+        <v>15698483.5698</v>
       </c>
     </row>
     <row r="50" s="37" customFormat="1" spans="1:15">
@@ -29849,7 +29889,7 @@
       </c>
       <c r="H50" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H50</f>
-        <v>692555.2367</v>
+        <v>1427835.2688</v>
       </c>
       <c r="I50" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I50</f>
@@ -29877,7 +29917,7 @@
       </c>
       <c r="O50" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O50</f>
-        <v>4218986.3419</v>
+        <v>4954266.374</v>
       </c>
     </row>
     <row r="51" s="37" customFormat="1" spans="1:15">
@@ -29911,7 +29951,7 @@
       </c>
       <c r="H51" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H51</f>
-        <v>0.304533666715811</v>
+        <v>0.310669180428351</v>
       </c>
       <c r="I51" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I51</f>
@@ -29939,7 +29979,7 @@
       </c>
       <c r="O51" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O51</f>
-        <v>0.315399688017098</v>
+        <v>0.315588849838387</v>
       </c>
     </row>
     <row r="52" s="37" customFormat="1" spans="1:15">
@@ -29973,7 +30013,7 @@
       </c>
       <c r="H52" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H52</f>
-        <v>0.635532809358435</v>
+        <v>0.622704199353945</v>
       </c>
       <c r="I52" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I52</f>
@@ -30001,7 +30041,7 @@
       </c>
       <c r="O52" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O52</f>
-        <v>0.650735294117647</v>
+        <v>0.645171056615198</v>
       </c>
     </row>
     <row r="53" s="37" customFormat="1" spans="1:15">
@@ -30035,7 +30075,7 @@
       </c>
       <c r="H53" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H53</f>
-        <v>0.189701330721307</v>
+        <v>0.172379549222688</v>
       </c>
       <c r="I53" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I53</f>
@@ -30063,7 +30103,7 @@
       </c>
       <c r="O53" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O53</f>
-        <v>0.181202712700823</v>
+        <v>0.177471830060303</v>
       </c>
     </row>
     <row r="54" s="37" customFormat="1" spans="1:15">
@@ -30097,7 +30137,7 @@
       </c>
       <c r="H54" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H54</f>
-        <v>12941.37</v>
+        <v>25673.18</v>
       </c>
       <c r="I54" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I54</f>
@@ -30125,7 +30165,7 @@
       </c>
       <c r="O54" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O54</f>
-        <v>146515.24</v>
+        <v>159247.05</v>
       </c>
     </row>
     <row r="55" s="37" customFormat="1" spans="1:15">
@@ -30159,7 +30199,7 @@
       </c>
       <c r="H55" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H55</f>
-        <v>623</v>
+        <v>1181</v>
       </c>
       <c r="I55" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I55</f>
@@ -30187,7 +30227,7 @@
       </c>
       <c r="O55" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O55</f>
-        <v>17199</v>
+        <v>17757</v>
       </c>
     </row>
     <row r="56" s="37" customFormat="1" spans="1:15">
@@ -30221,7 +30261,7 @@
       </c>
       <c r="H56" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H56</f>
-        <v>255</v>
+        <v>508</v>
       </c>
       <c r="I56" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I56</f>
@@ -30249,7 +30289,7 @@
       </c>
       <c r="O56" s="1">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O56</f>
-        <v>6281</v>
+        <v>6534</v>
       </c>
     </row>
     <row r="57" s="37" customFormat="1" spans="1:15">
@@ -30283,7 +30323,7 @@
       </c>
       <c r="H57" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H57</f>
-        <v>239297.004</v>
+        <v>1477637.646</v>
       </c>
       <c r="I57" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I57</f>
@@ -30311,7 +30351,7 @@
       </c>
       <c r="O57" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O57</f>
-        <v>6044804.1153</v>
+        <v>7283144.7573</v>
       </c>
     </row>
     <row r="58" s="37" customFormat="1" spans="1:15">
@@ -30345,7 +30385,7 @@
       </c>
       <c r="H58" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H58</f>
-        <v>80592.046</v>
+        <v>160215.761</v>
       </c>
       <c r="I58" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I58</f>
@@ -30373,7 +30413,7 @@
       </c>
       <c r="O58" s="21">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O58</f>
-        <v>2385818.1457</v>
+        <v>2465441.8607</v>
       </c>
     </row>
     <row r="59" s="37" customFormat="1" spans="1:15">
@@ -30407,7 +30447,7 @@
       </c>
       <c r="H59" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H59</f>
-        <v>0.336786690400854</v>
+        <v>0.108426962072676</v>
       </c>
       <c r="I59" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I59</f>
@@ -30435,7 +30475,7 @@
       </c>
       <c r="O59" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O59</f>
-        <v>0.394689075144926</v>
+        <v>0.338513367900432</v>
       </c>
     </row>
     <row r="60" s="37" customFormat="1" spans="1:15">
@@ -30469,7 +30509,7 @@
       </c>
       <c r="H60" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H60</f>
-        <v>0.590690208667737</v>
+        <v>0.569856054191363</v>
       </c>
       <c r="I60" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I60</f>
@@ -30497,7 +30537,7 @@
       </c>
       <c r="O60" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O60</f>
-        <v>0.634804349090063</v>
+        <v>0.632032437911809</v>
       </c>
     </row>
     <row r="61" s="37" customFormat="1" spans="1:15">
@@ -30531,7 +30571,7 @@
       </c>
       <c r="H61" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H61</f>
-        <v>0.160578749917827</v>
+        <v>0.160241288620787</v>
       </c>
       <c r="I61" s="13" t="e">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I61</f>
@@ -30559,7 +30599,7 @@
       </c>
       <c r="O61" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!O61</f>
-        <v>0.0614109001828437</v>
+        <v>0.0645916874124891</v>
       </c>
     </row>
     <row r="62" s="37" customFormat="1" spans="1:15">
@@ -37359,7 +37399,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ec3abd82-a414-4476-9a74-8fd433f846a7}</x14:id>
+          <x14:id>{11b2dc0e-f4e2-4b11-b795-6a8ea36cc53e}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37373,7 +37413,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ad81e660-adb2-4c44-ba2c-cb32f9409e11}</x14:id>
+          <x14:id>{8e06d658-4f0f-4241-91e6-58abea868049}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37387,7 +37427,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{dc93f3a9-c583-4f29-9b0d-8667fe64ced6}</x14:id>
+          <x14:id>{2c0bc188-d780-430e-919a-f63eaf2d0a9e}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37401,7 +37441,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{64e19edc-281a-492c-9bfa-5757f6d7f4b3}</x14:id>
+          <x14:id>{19dd85de-6207-4cac-b87a-1a59978c649b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37415,7 +37455,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6eb20218-6da8-449d-88a5-4c7cfee3a9d3}</x14:id>
+          <x14:id>{c0a87b2a-dc78-4f7c-97f6-988e40aa300e}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37429,7 +37469,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{880c0b46-21ed-470c-afb5-5b57a55fa534}</x14:id>
+          <x14:id>{fc5b717a-ec21-4adf-9a52-3f0a027f6a27}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37449,7 +37489,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{789db2cc-577d-46b2-9e87-1836ad337da8}</x14:id>
+          <x14:id>{c7f8a1e3-6e75-474f-927c-882a93369368}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37463,7 +37503,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{82437995-34b7-43b9-87c1-de075b1b2394}</x14:id>
+          <x14:id>{7262b42b-44a0-4f27-86ac-fcd42ea53b71}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37477,7 +37517,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0d56f005-0198-4d6a-896f-dc64e377ca60}</x14:id>
+          <x14:id>{7ad9ae39-1eb2-44e6-a172-78f00cbe2030}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37491,7 +37531,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{eae55dd0-f6e8-480a-8346-b42e42b5c8a8}</x14:id>
+          <x14:id>{62c313d3-9fbf-4429-8004-239336062e32}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37505,7 +37545,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{592992a1-831f-4749-977b-7b9b7456c46f}</x14:id>
+          <x14:id>{9fd94e65-dd54-418d-b2ae-a64ebd857edb}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37519,7 +37559,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0e07c3e9-066f-4ed7-aa44-dae1e91b4b47}</x14:id>
+          <x14:id>{82491f1e-24eb-4394-8f09-5dcee01b6beb}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37541,7 +37581,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{72c4bac1-3e03-46f5-8ae2-4eb5bfa9a360}</x14:id>
+          <x14:id>{78323c8a-698a-4008-8d47-a2e7b9aecb70}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37571,7 +37611,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0d83b2f4-558d-4203-b5ef-349d2d341b26}</x14:id>
+          <x14:id>{c297036d-285e-4e4f-9de4-1021a7c8da07}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37601,7 +37641,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{b4934688-0cf8-4319-92ff-35372a11c2e1}</x14:id>
+          <x14:id>{dfa5d315-8d46-402d-b669-95099a184466}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37631,7 +37671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{fd126515-fd4a-43f8-b379-92abd763a227}</x14:id>
+          <x14:id>{5810c1e8-6f6e-4fc3-a16e-f8ffef564445}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37661,7 +37701,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{cbd28c9e-25b7-422c-bf8c-0e3f9f21b031}</x14:id>
+          <x14:id>{52ed7f06-9a03-4508-a35c-92328d303115}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37691,7 +37731,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{57ee7dcb-df9c-462e-b650-0c321a1be40f}</x14:id>
+          <x14:id>{003dc371-8c46-48e5-bb82-0bc9832e2718}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37713,7 +37753,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1b2198fe-2011-4d5f-83eb-5132685df21e}</x14:id>
+          <x14:id>{7986bc79-5ed6-4121-8404-46757409e60b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37735,7 +37775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{85bbce98-7e23-4a66-8a4d-f6b6ed0b9cb0}</x14:id>
+          <x14:id>{2b87f753-36f0-4332-a28d-e3d507c5bc84}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37757,7 +37797,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d2a8b3d2-a6a0-416a-b85b-31083ae501d5}</x14:id>
+          <x14:id>{2699fb2c-c4dc-4e4e-8bea-099037fd348e}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37779,7 +37819,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0364943d-d06f-4c37-be88-7826407e9695}</x14:id>
+          <x14:id>{84950ce3-69ac-4bf1-8b0e-b035c49af64c}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37801,7 +37841,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{fe4eb5b9-8f9a-47a6-9f2b-b227c6f9b927}</x14:id>
+          <x14:id>{16770792-f1a6-4073-b131-1de1a3583af5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37823,7 +37863,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{57b11a37-fa9f-428a-abd8-4e99ba3f00e7}</x14:id>
+          <x14:id>{3954aa38-59ff-4a55-9e6a-df5e87e13e16}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37845,7 +37885,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d147febf-3e2b-433b-a7c6-0d3aeb3dc7b6}</x14:id>
+          <x14:id>{ec89d09a-7122-4ffb-80f1-f7ce4b2b3af0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37867,7 +37907,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{61384d78-5d07-49fe-ad7c-a44ce1ab1163}</x14:id>
+          <x14:id>{a5da7186-9f45-4f78-9c1d-66ca6f3438be}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37889,7 +37929,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{d43cbea3-e695-4982-b6c4-7eabfd694c43}</x14:id>
+          <x14:id>{d83863fa-282f-4adb-ba16-b33f4a6a3cdb}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37911,7 +37951,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{712d799c-ce57-4f15-98a6-cbea8ce88d04}</x14:id>
+          <x14:id>{6ad7ebd5-ce15-4605-b6a0-cd37b57e3924}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37933,7 +37973,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ba9210c7-4e29-47d2-a335-0718d03f238c}</x14:id>
+          <x14:id>{297d3cb0-18b0-413a-99a5-2161f6fd36d5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37955,7 +37995,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{82d0d6e6-6736-44e8-a09d-47f777db27ad}</x14:id>
+          <x14:id>{f5f1a0a5-754f-4d90-813f-dc4359d3b52b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37977,7 +38017,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{02256ed3-46bd-4d20-9ab3-d19c36967293}</x14:id>
+          <x14:id>{ce8fffbd-1ae9-47e9-b0e4-a9f7e53589d6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -37999,7 +38039,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{dbe685ab-7d2b-4a12-abd6-80ecc8eaf52d}</x14:id>
+          <x14:id>{1a76a20b-080a-4138-9a29-0d927a5ee620}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38018,7 +38058,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ec3abd82-a414-4476-9a74-8fd433f846a7}">
+          <x14:cfRule type="dataBar" id="{11b2dc0e-f4e2-4b11-b795-6a8ea36cc53e}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38031,7 +38071,7 @@
           <xm:sqref>C8:O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ad81e660-adb2-4c44-ba2c-cb32f9409e11}">
+          <x14:cfRule type="dataBar" id="{8e06d658-4f0f-4241-91e6-58abea868049}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38044,7 +38084,7 @@
           <xm:sqref>C12:O12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{dc93f3a9-c583-4f29-9b0d-8667fe64ced6}">
+          <x14:cfRule type="dataBar" id="{2c0bc188-d780-430e-919a-f63eaf2d0a9e}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38057,7 +38097,7 @@
           <xm:sqref>C16:O16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{64e19edc-281a-492c-9bfa-5757f6d7f4b3}">
+          <x14:cfRule type="dataBar" id="{19dd85de-6207-4cac-b87a-1a59978c649b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38070,7 +38110,7 @@
           <xm:sqref>C20:O20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6eb20218-6da8-449d-88a5-4c7cfee3a9d3}">
+          <x14:cfRule type="dataBar" id="{c0a87b2a-dc78-4f7c-97f6-988e40aa300e}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38083,7 +38123,7 @@
           <xm:sqref>C24:O24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{880c0b46-21ed-470c-afb5-5b57a55fa534}">
+          <x14:cfRule type="dataBar" id="{fc5b717a-ec21-4adf-9a52-3f0a027f6a27}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38096,7 +38136,7 @@
           <xm:sqref>O26</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{789db2cc-577d-46b2-9e87-1836ad337da8}">
+          <x14:cfRule type="dataBar" id="{c7f8a1e3-6e75-474f-927c-882a93369368}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38109,7 +38149,7 @@
           <xm:sqref>C27:O27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{82437995-34b7-43b9-87c1-de075b1b2394}">
+          <x14:cfRule type="dataBar" id="{7262b42b-44a0-4f27-86ac-fcd42ea53b71}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38122,7 +38162,7 @@
           <xm:sqref>C36:O36</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0d56f005-0198-4d6a-896f-dc64e377ca60}">
+          <x14:cfRule type="dataBar" id="{7ad9ae39-1eb2-44e6-a172-78f00cbe2030}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38135,7 +38175,7 @@
           <xm:sqref>C44:O44</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{eae55dd0-f6e8-480a-8346-b42e42b5c8a8}">
+          <x14:cfRule type="dataBar" id="{62c313d3-9fbf-4429-8004-239336062e32}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38148,7 +38188,7 @@
           <xm:sqref>C52:O52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{592992a1-831f-4749-977b-7b9b7456c46f}">
+          <x14:cfRule type="dataBar" id="{9fd94e65-dd54-418d-b2ae-a64ebd857edb}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38161,7 +38201,7 @@
           <xm:sqref>C60:O60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0e07c3e9-066f-4ed7-aa44-dae1e91b4b47}">
+          <x14:cfRule type="dataBar" id="{82491f1e-24eb-4394-8f09-5dcee01b6beb}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38174,7 +38214,7 @@
           <xm:sqref>C124:O124</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{72c4bac1-3e03-46f5-8ae2-4eb5bfa9a360}">
+          <x14:cfRule type="dataBar" id="{78323c8a-698a-4008-8d47-a2e7b9aecb70}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38187,7 +38227,7 @@
           <xm:sqref>C26:N26 D27:N27 C28:O28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0d83b2f4-558d-4203-b5ef-349d2d341b26}">
+          <x14:cfRule type="dataBar" id="{c297036d-285e-4e4f-9de4-1021a7c8da07}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38200,7 +38240,7 @@
           <xm:sqref>C35:N35 D36:N36 C37:O37</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{b4934688-0cf8-4319-92ff-35372a11c2e1}">
+          <x14:cfRule type="dataBar" id="{dfa5d315-8d46-402d-b669-95099a184466}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38213,7 +38253,7 @@
           <xm:sqref>C43:N43 D44:N44 C45:O45</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{fd126515-fd4a-43f8-b379-92abd763a227}">
+          <x14:cfRule type="dataBar" id="{5810c1e8-6f6e-4fc3-a16e-f8ffef564445}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38226,7 +38266,7 @@
           <xm:sqref>C51:N51 D52:N52 C53:O53</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{cbd28c9e-25b7-422c-bf8c-0e3f9f21b031}">
+          <x14:cfRule type="dataBar" id="{52ed7f06-9a03-4508-a35c-92328d303115}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38239,7 +38279,7 @@
           <xm:sqref>C59:N59 D60:N60 C61:O61</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{57ee7dcb-df9c-462e-b650-0c321a1be40f}">
+          <x14:cfRule type="dataBar" id="{003dc371-8c46-48e5-bb82-0bc9832e2718}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38252,7 +38292,7 @@
           <xm:sqref>C67:N67 D68:N68 C69:O69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1b2198fe-2011-4d5f-83eb-5132685df21e}">
+          <x14:cfRule type="dataBar" id="{7986bc79-5ed6-4121-8404-46757409e60b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38265,7 +38305,7 @@
           <xm:sqref>C68:O68 D69:N69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{85bbce98-7e23-4a66-8a4d-f6b6ed0b9cb0}">
+          <x14:cfRule type="dataBar" id="{2b87f753-36f0-4332-a28d-e3d507c5bc84}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38278,7 +38318,7 @@
           <xm:sqref>C75:N75 D76:N76 C77:O77</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d2a8b3d2-a6a0-416a-b85b-31083ae501d5}">
+          <x14:cfRule type="dataBar" id="{2699fb2c-c4dc-4e4e-8bea-099037fd348e}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38291,7 +38331,7 @@
           <xm:sqref>C76:O76 D77:N77</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0364943d-d06f-4c37-be88-7826407e9695}">
+          <x14:cfRule type="dataBar" id="{84950ce3-69ac-4bf1-8b0e-b035c49af64c}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38304,7 +38344,7 @@
           <xm:sqref>C83:N83 D84:N84 C85:O85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{fe4eb5b9-8f9a-47a6-9f2b-b227c6f9b927}">
+          <x14:cfRule type="dataBar" id="{16770792-f1a6-4073-b131-1de1a3583af5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38317,7 +38357,7 @@
           <xm:sqref>C84:O84 D85:N85</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{57b11a37-fa9f-428a-abd8-4e99ba3f00e7}">
+          <x14:cfRule type="dataBar" id="{3954aa38-59ff-4a55-9e6a-df5e87e13e16}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38330,7 +38370,7 @@
           <xm:sqref>C91:N91 D92:N92 C93:O93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d147febf-3e2b-433b-a7c6-0d3aeb3dc7b6}">
+          <x14:cfRule type="dataBar" id="{ec89d09a-7122-4ffb-80f1-f7ce4b2b3af0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38343,7 +38383,7 @@
           <xm:sqref>C92:O92 D93:N93</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{61384d78-5d07-49fe-ad7c-a44ce1ab1163}">
+          <x14:cfRule type="dataBar" id="{a5da7186-9f45-4f78-9c1d-66ca6f3438be}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38356,7 +38396,7 @@
           <xm:sqref>C99:N99 D100:N100 C101:O101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{d43cbea3-e695-4982-b6c4-7eabfd694c43}">
+          <x14:cfRule type="dataBar" id="{d83863fa-282f-4adb-ba16-b33f4a6a3cdb}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38369,7 +38409,7 @@
           <xm:sqref>C100:O100 D101:N101</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{712d799c-ce57-4f15-98a6-cbea8ce88d04}">
+          <x14:cfRule type="dataBar" id="{6ad7ebd5-ce15-4605-b6a0-cd37b57e3924}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38382,7 +38422,7 @@
           <xm:sqref>C107:N107 D108:N108 C109:O109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ba9210c7-4e29-47d2-a335-0718d03f238c}">
+          <x14:cfRule type="dataBar" id="{297d3cb0-18b0-413a-99a5-2161f6fd36d5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38395,7 +38435,7 @@
           <xm:sqref>C108:O108 D109:N109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{82d0d6e6-6736-44e8-a09d-47f777db27ad}">
+          <x14:cfRule type="dataBar" id="{f5f1a0a5-754f-4d90-813f-dc4359d3b52b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38408,7 +38448,7 @@
           <xm:sqref>C115:N115 D116:N116 C117:O117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{02256ed3-46bd-4d20-9ab3-d19c36967293}">
+          <x14:cfRule type="dataBar" id="{ce8fffbd-1ae9-47e9-b0e4-a9f7e53589d6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -38421,7 +38461,7 @@
           <xm:sqref>C116:O116 D117:N117</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{dbe685ab-7d2b-4a12-abd6-80ecc8eaf52d}">
+          <x14:cfRule type="dataBar" id="{1a76a20b-080a-4138-9a29-0d927a5ee620}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -44498,7 +44538,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="3">
         <f>(F7+G7+H7)</f>
-        <v>1003976.28</v>
+        <v>1188871.27</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -44536,7 +44576,7 @@
       <c r="E5" s="5"/>
       <c r="F5" s="6">
         <f>(F7+G7+H7)/(F6+G6+H6)</f>
-        <v>0.96637899787671</v>
+        <v>1.14434997060589</v>
       </c>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -44651,7 +44691,7 @@
       </c>
       <c r="H7" s="12">
         <f>'[2]2026年月度数据汇总--俄罗斯'!H3+'[2]2026年月度数据汇总--俄罗斯'!H8</f>
-        <v>180718.61</v>
+        <v>365613.6</v>
       </c>
       <c r="I7" s="12">
         <f>'[2]2026年月度数据汇总--俄罗斯'!I3+'[2]2026年月度数据汇总--俄罗斯'!I8</f>
@@ -44679,7 +44719,7 @@
       </c>
       <c r="O7" s="12">
         <f t="shared" si="0"/>
-        <v>2526250.95</v>
+        <v>2711145.94</v>
       </c>
     </row>
     <row r="8" ht="15.6" spans="1:15">
@@ -44713,7 +44753,7 @@
       </c>
       <c r="H8" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H8</f>
-        <v>0.535748473942456</v>
+        <v>1.05062851406593</v>
       </c>
       <c r="I8" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I8</f>
@@ -44741,7 +44781,7 @@
       </c>
       <c r="O8" s="20">
         <f>O7/O6</f>
-        <v>0.443929943639255</v>
+        <v>0.476420944776684</v>
       </c>
     </row>
     <row r="9" ht="15.6" spans="1:15">
@@ -44899,7 +44939,7 @@
       </c>
       <c r="H11" s="11">
         <f>'[2]2026年月度数据汇总--俄罗斯'!H4+'[2]2026年月度数据汇总--俄罗斯'!H9</f>
-        <v>9793</v>
+        <v>20745</v>
       </c>
       <c r="I11" s="11">
         <f>'[2]2026年月度数据汇总--俄罗斯'!I4+'[2]2026年月度数据汇总--俄罗斯'!I9</f>
@@ -44927,7 +44967,7 @@
       </c>
       <c r="O11" s="11">
         <f t="shared" si="0"/>
-        <v>120172</v>
+        <v>131124</v>
       </c>
     </row>
     <row r="12" ht="15.6" spans="1:15">
@@ -44961,7 +45001,7 @@
       </c>
       <c r="H12" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H12</f>
-        <v>0.395130201208745</v>
+        <v>0.814808366702315</v>
       </c>
       <c r="I12" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I12</f>
@@ -44989,7 +45029,7 @@
       </c>
       <c r="O12" s="20">
         <f>O11/O10</f>
-        <v>0.320764890215192</v>
+        <v>0.349998131549586</v>
       </c>
     </row>
     <row r="13" ht="15.6" spans="1:15">
@@ -45147,7 +45187,7 @@
       </c>
       <c r="H15" s="11">
         <f>'[2]2026年月度数据汇总--俄罗斯'!H5+'[2]2026年月度数据汇总--俄罗斯'!H10</f>
-        <v>3251</v>
+        <v>6862</v>
       </c>
       <c r="I15" s="11">
         <f>'[2]2026年月度数据汇总--俄罗斯'!I5+'[2]2026年月度数据汇总--俄罗斯'!I10</f>
@@ -45175,7 +45215,7 @@
       </c>
       <c r="O15" s="11">
         <f>SUM(C15:N15)</f>
-        <v>42595</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="16" ht="15.6" spans="1:15">
@@ -45209,7 +45249,7 @@
       </c>
       <c r="H16" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H16</f>
-        <v>0.441264841541795</v>
+        <v>0.919275009888344</v>
       </c>
       <c r="I16" s="13">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I16</f>
@@ -45237,7 +45277,7 @@
       </c>
       <c r="O16" s="20">
         <f>O15/O14</f>
-        <v>0.366758734489063</v>
+        <v>0.397850782622412</v>
       </c>
     </row>
     <row r="17" ht="15.6" spans="1:15">
@@ -45395,7 +45435,7 @@
       </c>
       <c r="H19" s="19">
         <f>'[2]2026年月度数据汇总--俄罗斯'!H6+'[2]2026年月度数据汇总--俄罗斯'!H11</f>
-        <v>4145841.474</v>
+        <v>9012496.5492</v>
       </c>
       <c r="I19" s="19">
         <f>'[2]2026年月度数据汇总--俄罗斯'!I6+'[2]2026年月度数据汇总--俄罗斯'!I11</f>
@@ -45423,7 +45463,7 @@
       </c>
       <c r="O19" s="19">
         <f>SUM(C19:N19)</f>
-        <v>48155870.5875</v>
+        <v>53022525.6627</v>
       </c>
     </row>
     <row r="20" ht="15.6" spans="1:15">
@@ -45457,7 +45497,7 @@
       </c>
       <c r="H20" s="20">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!H20</f>
-        <v>0.476369032961964</v>
+        <v>1.07917936735439</v>
       </c>
       <c r="I20" s="20">
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!I20</f>
@@ -45485,7 +45525,7 @@
       </c>
       <c r="O20" s="20">
         <f>O19/O18</f>
-        <v>0.0295088919321862</v>
+        <v>0.0324910745183023</v>
       </c>
     </row>
     <row r="21" ht="15.6" spans="1:15">
@@ -45559,21 +45599,57 @@
         <f>'[2]2026年度男装数据汇总分析--俄罗斯'!B22</f>
         <v>GSV目标</v>
       </c>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="21"/>
-      <c r="L22" s="21"/>
-      <c r="M22" s="21"/>
-      <c r="N22" s="21"/>
+      <c r="C22" s="21">
+        <f>C18*(1-0.68)/12.5</f>
+        <v>2376622.08</v>
+      </c>
+      <c r="D22" s="21">
+        <f t="shared" ref="D22:N22" si="1">D18*(1-0.68)/12.5</f>
+        <v>2637926.4</v>
+      </c>
+      <c r="E22" s="21">
+        <f t="shared" si="1"/>
+        <v>2515968</v>
+      </c>
+      <c r="F22" s="21">
+        <f t="shared" si="1"/>
+        <v>2420480</v>
+      </c>
+      <c r="G22" s="21">
+        <f t="shared" si="1"/>
+        <v>2507520</v>
+      </c>
+      <c r="H22" s="21">
+        <f t="shared" si="1"/>
+        <v>2751252.48</v>
+      </c>
+      <c r="I22" s="21">
+        <f t="shared" si="1"/>
+        <v>3913955.84</v>
+      </c>
+      <c r="J22" s="21">
+        <f t="shared" si="1"/>
+        <v>4512000</v>
+      </c>
+      <c r="K22" s="21">
+        <f t="shared" si="1"/>
+        <v>4833024</v>
+      </c>
+      <c r="L22" s="21">
+        <f t="shared" si="1"/>
+        <v>5015040</v>
+      </c>
+      <c r="M22" s="21">
+        <f t="shared" si="1"/>
+        <v>4840960</v>
+      </c>
+      <c r="N22" s="21">
+        <f t="shared" si="1"/>
+        <v>3452160</v>
+      </c>
       <c r="O22" s="28">
         <f>SUM(C22:N22)</f>
-        <v>0</v>
+        <v>41776908.8</v>
       </c>
     </row>
     <row r="23" ht="15.6" spans="1:15">
@@ -45623,9 +45699,9 @@
       <c r="L24" s="13"/>
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
-      <c r="O24" s="20" t="e">
+      <c r="O24" s="20">
         <f>O23/O22</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" ht="15.6" spans="1:15">
@@ -45700,55 +45776,55 @@
         <v>退款率</v>
       </c>
       <c r="C26" s="13">
-        <f t="shared" ref="C26:O26" si="1">1-C23/C19</f>
+        <f t="shared" ref="C26:O26" si="2">1-C23/C19</f>
         <v>1</v>
       </c>
       <c r="D26" s="13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="E26" s="13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="F26" s="13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="G26" s="13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="H26" s="13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="I26" s="13" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="J26" s="13" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="K26" s="13" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="L26" s="13" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="M26" s="13" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="N26" s="13" t="e">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O26" s="13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
@@ -45762,56 +45838,56 @@
         <v>退货率</v>
       </c>
       <c r="C27" s="13">
-        <f t="shared" ref="C27:O27" si="2">1-C15/C11</f>
+        <f t="shared" ref="C27:O27" si="3">1-C15/C11</f>
         <v>0.65554314437308</v>
       </c>
       <c r="D27" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.640546006066734</v>
       </c>
       <c r="E27" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.626170547774923</v>
       </c>
       <c r="F27" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.632716432741274</v>
       </c>
       <c r="G27" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.672910491997629</v>
       </c>
       <c r="H27" s="13">
-        <f t="shared" si="2"/>
-        <v>0.668028183396304</v>
+        <f t="shared" si="3"/>
+        <v>0.669221499156423</v>
       </c>
       <c r="I27" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="J27" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="K27" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="L27" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="M27" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="N27" s="13" t="e">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O27" s="13">
-        <f t="shared" si="2"/>
-        <v>0.645549712079353</v>
+        <f t="shared" si="3"/>
+        <v>0.647615997071474</v>
       </c>
     </row>
     <row r="28" ht="15.6" spans="1:15">
@@ -45824,55 +45900,55 @@
         <v>利润率</v>
       </c>
       <c r="C28" s="13" t="e">
-        <f t="shared" ref="C28:O28" si="3">C7/(C23)</f>
+        <f t="shared" ref="C28:O28" si="4">C7/(C23)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="D28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="E28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="F28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="G28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="H28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="J28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="K28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="L28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="M28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="N28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O28" s="13" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -45990,7 +46066,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{cde86fa1-159c-4f03-8e1a-6d876c3c85f6}</x14:id>
+          <x14:id>{db02600c-d341-4ddd-8277-7fe6e91d271d}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46004,7 +46080,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9dfc139c-9a0e-4699-9712-f5c541e7a679}</x14:id>
+          <x14:id>{59d50552-5b6d-494b-86be-c7f6ac1aea44}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46018,7 +46094,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{40988baa-ef10-4184-8dc0-a79b419fd26c}</x14:id>
+          <x14:id>{22bac7bf-1518-4fcd-afb1-3e6628cb6a86}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46032,7 +46108,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{589abc33-40db-47a9-925e-6b290718afbb}</x14:id>
+          <x14:id>{ca03ff5e-323a-476f-b135-89634bd4b671}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46046,7 +46122,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{00e2b72e-ba39-462b-9cad-45299ead12da}</x14:id>
+          <x14:id>{45dda5cc-5576-4b68-8ad5-b3da92a33120}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46060,7 +46136,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{325d8e3e-5d02-4469-8646-84309071d266}</x14:id>
+          <x14:id>{97937f43-5af6-4447-87fc-08c5022c1bc8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46074,7 +46150,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{b048b597-4661-45f6-b155-aa34f7092ccf}</x14:id>
+          <x14:id>{847c7803-8fce-4168-90db-cc0590b24295}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46088,7 +46164,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9e071a33-8785-49fa-9546-18fdd230ec1d}</x14:id>
+          <x14:id>{54b17f45-da40-4180-a64f-a65310d67a93}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46102,7 +46178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{85051f7f-ffe2-4e0d-809b-d9a28e04f24b}</x14:id>
+          <x14:id>{954ea273-1b08-4cc0-a6da-a5c0a8aaf9cc}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46116,7 +46192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{138d7ac8-eaf5-4788-bd0c-3ef3ac1277b1}</x14:id>
+          <x14:id>{6485c2aa-4451-48b8-879a-7a2bf4882b33}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46130,7 +46206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5108c85e-836c-4c7e-9698-72934ea23f58}</x14:id>
+          <x14:id>{b9050113-e4c3-427d-82ce-fc0bed9030a1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46166,7 +46242,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{05b5708c-e55f-448d-9fe0-0afe6eeae5c4}</x14:id>
+          <x14:id>{f1638b27-1922-4e80-9eb1-fd469f698201}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -46185,7 +46261,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{cde86fa1-159c-4f03-8e1a-6d876c3c85f6}">
+          <x14:cfRule type="dataBar" id="{db02600c-d341-4ddd-8277-7fe6e91d271d}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46198,7 +46274,7 @@
           <xm:sqref>C8:N8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9dfc139c-9a0e-4699-9712-f5c541e7a679}">
+          <x14:cfRule type="dataBar" id="{59d50552-5b6d-494b-86be-c7f6ac1aea44}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46211,7 +46287,7 @@
           <xm:sqref>O8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{40988baa-ef10-4184-8dc0-a79b419fd26c}">
+          <x14:cfRule type="dataBar" id="{22bac7bf-1518-4fcd-afb1-3e6628cb6a86}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46224,7 +46300,7 @@
           <xm:sqref>C12:N12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{589abc33-40db-47a9-925e-6b290718afbb}">
+          <x14:cfRule type="dataBar" id="{ca03ff5e-323a-476f-b135-89634bd4b671}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46237,7 +46313,7 @@
           <xm:sqref>O12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{00e2b72e-ba39-462b-9cad-45299ead12da}">
+          <x14:cfRule type="dataBar" id="{45dda5cc-5576-4b68-8ad5-b3da92a33120}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46250,7 +46326,7 @@
           <xm:sqref>C16:N16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{325d8e3e-5d02-4469-8646-84309071d266}">
+          <x14:cfRule type="dataBar" id="{97937f43-5af6-4447-87fc-08c5022c1bc8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46263,7 +46339,7 @@
           <xm:sqref>O16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{b048b597-4661-45f6-b155-aa34f7092ccf}">
+          <x14:cfRule type="dataBar" id="{847c7803-8fce-4168-90db-cc0590b24295}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46276,7 +46352,7 @@
           <xm:sqref>B20:N20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9e071a33-8785-49fa-9546-18fdd230ec1d}">
+          <x14:cfRule type="dataBar" id="{54b17f45-da40-4180-a64f-a65310d67a93}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46289,7 +46365,7 @@
           <xm:sqref>O20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{85051f7f-ffe2-4e0d-809b-d9a28e04f24b}">
+          <x14:cfRule type="dataBar" id="{954ea273-1b08-4cc0-a6da-a5c0a8aaf9cc}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46302,7 +46378,7 @@
           <xm:sqref>C24:N24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{138d7ac8-eaf5-4788-bd0c-3ef3ac1277b1}">
+          <x14:cfRule type="dataBar" id="{6485c2aa-4451-48b8-879a-7a2bf4882b33}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46315,7 +46391,7 @@
           <xm:sqref>O24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5108c85e-836c-4c7e-9698-72934ea23f58}">
+          <x14:cfRule type="dataBar" id="{b9050113-e4c3-427d-82ce-fc0bed9030a1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46328,7 +46404,7 @@
           <xm:sqref>C27:O27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{05b5708c-e55f-448d-9fe0-0afe6eeae5c4}">
+          <x14:cfRule type="dataBar" id="{f1638b27-1922-4e80-9eb1-fd469f698201}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -46348,6 +46424,7 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <NetdiskSupbooks xmlns="http://www.wps.cn/et/2019/netdiskSupbooks">
+  <NetdiskSupbook Target="file:///C:\Users\12139\WPSDrive\1725300681\WPS企业云盘\瑞安市水滴电子商务有限公司\团队文档\俄罗斯运营二部\梦瑶\2026WB年规进度-梦瑶.xlsx" FileId="497856789952" NetdiskName="yunwps"/>
   <NetdiskSupbook Target="file:///C:\Users\12139\WPSDrive\1725300681\WPS企业云盘\瑞安市水滴电子商务有限公司\团队文档\俄罗斯运营一部\WB运营报表\目标\2026年俄罗斯一部目标拆分.xlsx" FileId="505692420986" NetdiskName="yunwps"/>
 </NetdiskSupbooks>
 </file>

</xml_diff>